<commit_message>
Add cocktail, cafe and liquid-mix lines to the order guide
Expand the workbook from 20 to 40 product lines across seven sections:
smoothie powder prep (Amazon and other vendors), smoothie liquid mix,
cocktail/bar prep, cafe, unassigned, and in-house.

Lines with recipe usage mapped calculate packs per cycle as before;
the cocktail, cafe and liquid-mix lines show "par" instead, since no
grams-per-cycle exist for them yet, and remain orderable by hand.

Add a Bar Prep Reference tab listing the 23 TH - Bar Prep recipes in
Margin Edge so those lines can be made recipe-driven later. Three of
them had ingredients pulled, confirming loose leaf chai feeds Brewed
Chai Tea and coconut cream feeds both Fall Coconut Cream and the Being
Brigid Liquid Mix.

Add flags for products Margin Edge prices at zero and for the Columbus
water cost appearing in bar recipes too.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01W5WUQdsyFygtfJrtmcjz3J
</commit_message>
<xml_diff>
--- a/order-guide/TownHall-Order-Guide.xlsx
+++ b/order-guide/TownHall-Order-Guide.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Recipe Usage" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Order Guide" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Notes &amp; Flags" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Other Categories" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Bar Prep Reference" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23,7 +23,7 @@
     <numFmt numFmtId="164" formatCode="$#,##0.00;($#,##0.00);-"/>
     <numFmt numFmtId="165" formatCode="$0.0000"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="18">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -104,8 +104,20 @@
     </font>
     <font>
       <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00808080"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <b val="1"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00808080"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -166,7 +178,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -189,7 +201,9 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="11" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -204,15 +218,18 @@
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="14" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="15" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -222,8 +239,12 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
@@ -1052,13 +1073,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M38"/>
+  <dimension ref="A1:M63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="52" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
@@ -1067,20 +1088,20 @@
     <col width="11" customWidth="1" min="10" max="10"/>
     <col width="11" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="44" customWidth="1" min="13" max="13"/>
+    <col width="46" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="10" t="inlineStr">
         <is>
-          <t>TownHall — Smoothie Powder Prep Order Guide</t>
+          <t>TownHall — Order Guide</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Per location, per cycle (one batch of each of the four powder mixes). Columbus and Cleveland both run this prep — order for each site.</t>
+          <t>Per location, per cycle. Columbus and Cleveland both run this prep — order for each site.</t>
         </is>
       </c>
     </row>
@@ -1109,7 +1130,7 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Pack Size (g)</t>
+          <t>Pack Size</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -1161,7 +1182,7 @@
     <row r="6">
       <c r="A6" s="12" t="inlineStr">
         <is>
-          <t>AMAZON BUSINESS</t>
+          <t>SMOOTHIE POWDER PREP — AMAZON BUSINESS</t>
         </is>
       </c>
       <c r="B6" s="13" t="n"/>
@@ -1193,14 +1214,16 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D7" s="14" t="n">
-        <v>400</v>
+      <c r="D7" s="14" t="inlineStr">
+        <is>
+          <t>400 g</t>
+        </is>
       </c>
       <c r="E7" s="15" t="n">
         <v>28.25</v>
       </c>
       <c r="F7" s="16">
-        <f>IFERROR(E7/D7,"")</f>
+        <f>IFERROR(E7/400,"")</f>
         <v/>
       </c>
       <c r="G7" s="17">
@@ -1208,7 +1231,7 @@
         <v/>
       </c>
       <c r="H7" s="18">
-        <f>IFERROR(ROUNDUP(G7/D7,0),"")</f>
+        <f>IFERROR(ROUNDUP(G7/400,0),"")</f>
         <v/>
       </c>
       <c r="I7" s="19" t="n"/>
@@ -1243,14 +1266,16 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D8" s="14" t="n">
-        <v>400</v>
+      <c r="D8" s="14" t="inlineStr">
+        <is>
+          <t>400 g</t>
+        </is>
       </c>
       <c r="E8" s="15" t="n">
         <v>28.25</v>
       </c>
       <c r="F8" s="16">
-        <f>IFERROR(E8/D8,"")</f>
+        <f>IFERROR(E8/400,"")</f>
         <v/>
       </c>
       <c r="G8" s="17">
@@ -1258,7 +1283,7 @@
         <v/>
       </c>
       <c r="H8" s="18">
-        <f>IFERROR(ROUNDUP(G8/D8,0),"")</f>
+        <f>IFERROR(ROUNDUP(G8/400,0),"")</f>
         <v/>
       </c>
       <c r="I8" s="19" t="n"/>
@@ -1293,14 +1318,16 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D9" s="14" t="n">
-        <v>900</v>
+      <c r="D9" s="14" t="inlineStr">
+        <is>
+          <t>900 g</t>
+        </is>
       </c>
       <c r="E9" s="15" t="n">
         <v>84</v>
       </c>
       <c r="F9" s="16">
-        <f>IFERROR(E9/D9,"")</f>
+        <f>IFERROR(E9/900,"")</f>
         <v/>
       </c>
       <c r="G9" s="17">
@@ -1308,7 +1335,7 @@
         <v/>
       </c>
       <c r="H9" s="18">
-        <f>IFERROR(ROUNDUP(G9/D9,0),"")</f>
+        <f>IFERROR(ROUNDUP(G9/900,0),"")</f>
         <v/>
       </c>
       <c r="I9" s="19" t="n"/>
@@ -1343,14 +1370,16 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D10" s="14" t="n">
-        <v>243</v>
+      <c r="D10" s="14" t="inlineStr">
+        <is>
+          <t>243 g</t>
+        </is>
       </c>
       <c r="E10" s="15" t="n">
         <v>42.74</v>
       </c>
       <c r="F10" s="16">
-        <f>IFERROR(E10/D10,"")</f>
+        <f>IFERROR(E10/243,"")</f>
         <v/>
       </c>
       <c r="G10" s="17">
@@ -1358,7 +1387,7 @@
         <v/>
       </c>
       <c r="H10" s="18">
-        <f>IFERROR(ROUNDUP(G10/D10,0),"")</f>
+        <f>IFERROR(ROUNDUP(G10/243,0),"")</f>
         <v/>
       </c>
       <c r="I10" s="19" t="n"/>
@@ -1393,14 +1422,16 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D11" s="14" t="n">
-        <v>283</v>
+      <c r="D11" s="14" t="inlineStr">
+        <is>
+          <t>283 g</t>
+        </is>
       </c>
       <c r="E11" s="15" t="n">
         <v>25.34</v>
       </c>
       <c r="F11" s="16">
-        <f>IFERROR(E11/D11,"")</f>
+        <f>IFERROR(E11/283,"")</f>
         <v/>
       </c>
       <c r="G11" s="17">
@@ -1408,7 +1439,7 @@
         <v/>
       </c>
       <c r="H11" s="18">
-        <f>IFERROR(ROUNDUP(G11/D11,0),"")</f>
+        <f>IFERROR(ROUNDUP(G11/283,0),"")</f>
         <v/>
       </c>
       <c r="I11" s="19" t="n"/>
@@ -1443,14 +1474,16 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D12" s="14" t="n">
-        <v>1814</v>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
+          <t>1,814 g</t>
+        </is>
       </c>
       <c r="E12" s="15" t="n">
         <v>28.41</v>
       </c>
       <c r="F12" s="16">
-        <f>IFERROR(E12/D12,"")</f>
+        <f>IFERROR(E12/1814,"")</f>
         <v/>
       </c>
       <c r="G12" s="17">
@@ -1458,7 +1491,7 @@
         <v/>
       </c>
       <c r="H12" s="18">
-        <f>IFERROR(ROUNDUP(G12/D12,0),"")</f>
+        <f>IFERROR(ROUNDUP(G12/1814,0),"")</f>
         <v/>
       </c>
       <c r="I12" s="19" t="n"/>
@@ -1473,7 +1506,7 @@
       </c>
       <c r="M12" s="22" t="inlineStr">
         <is>
-          <t>UNSWEETENED ONLY. Do not substitute Lakanto (monk-fruit sweetened) — Keto has a separate monkfruit line.</t>
+          <t>UNSWEETENED ONLY. Do not substitute Lakanto — Keto has a separate monkfruit line.</t>
         </is>
       </c>
     </row>
@@ -1493,14 +1526,16 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D13" s="14" t="n">
-        <v>454</v>
+      <c r="D13" s="14" t="inlineStr">
+        <is>
+          <t>454 g</t>
+        </is>
       </c>
       <c r="E13" s="15" t="n">
         <v>16.29</v>
       </c>
       <c r="F13" s="16">
-        <f>IFERROR(E13/D13,"")</f>
+        <f>IFERROR(E13/454,"")</f>
         <v/>
       </c>
       <c r="G13" s="17">
@@ -1508,7 +1543,7 @@
         <v/>
       </c>
       <c r="H13" s="18">
-        <f>IFERROR(ROUNDUP(G13/D13,0),"")</f>
+        <f>IFERROR(ROUNDUP(G13/454,0),"")</f>
         <v/>
       </c>
       <c r="I13" s="19" t="n"/>
@@ -1539,14 +1574,16 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D14" s="14" t="n">
-        <v>100</v>
+      <c r="D14" s="14" t="inlineStr">
+        <is>
+          <t>100 g</t>
+        </is>
       </c>
       <c r="E14" s="15" t="n">
         <v>34.74</v>
       </c>
       <c r="F14" s="16">
-        <f>IFERROR(E14/D14,"")</f>
+        <f>IFERROR(E14/100,"")</f>
         <v/>
       </c>
       <c r="G14" s="17">
@@ -1554,7 +1591,7 @@
         <v/>
       </c>
       <c r="H14" s="18">
-        <f>IFERROR(ROUNDUP(G14/D14,0),"")</f>
+        <f>IFERROR(ROUNDUP(G14/100,0),"")</f>
         <v/>
       </c>
       <c r="I14" s="19" t="n"/>
@@ -1589,14 +1626,16 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D15" s="14" t="n">
-        <v>907</v>
+      <c r="D15" s="14" t="inlineStr">
+        <is>
+          <t>907 g</t>
+        </is>
       </c>
       <c r="E15" s="15" t="n">
         <v>23.35</v>
       </c>
       <c r="F15" s="16">
-        <f>IFERROR(E15/D15,"")</f>
+        <f>IFERROR(E15/907,"")</f>
         <v/>
       </c>
       <c r="G15" s="17">
@@ -1604,7 +1643,7 @@
         <v/>
       </c>
       <c r="H15" s="18">
-        <f>IFERROR(ROUNDUP(G15/D15,0),"")</f>
+        <f>IFERROR(ROUNDUP(G15/907,0),"")</f>
         <v/>
       </c>
       <c r="I15" s="19" t="n"/>
@@ -1639,14 +1678,16 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D16" s="14" t="n">
-        <v>454</v>
+      <c r="D16" s="14" t="inlineStr">
+        <is>
+          <t>454 g</t>
+        </is>
       </c>
       <c r="E16" s="15" t="n">
         <v>14.69</v>
       </c>
       <c r="F16" s="16">
-        <f>IFERROR(E16/D16,"")</f>
+        <f>IFERROR(E16/454,"")</f>
         <v/>
       </c>
       <c r="G16" s="17">
@@ -1654,7 +1695,7 @@
         <v/>
       </c>
       <c r="H16" s="18">
-        <f>IFERROR(ROUNDUP(G16/D16,0),"")</f>
+        <f>IFERROR(ROUNDUP(G16/454,0),"")</f>
         <v/>
       </c>
       <c r="I16" s="19" t="n"/>
@@ -1689,14 +1730,16 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D17" s="14" t="n">
-        <v>907</v>
+      <c r="D17" s="14" t="inlineStr">
+        <is>
+          <t>907 g</t>
+        </is>
       </c>
       <c r="E17" s="15" t="n">
         <v>13.97</v>
       </c>
       <c r="F17" s="16">
-        <f>IFERROR(E17/D17,"")</f>
+        <f>IFERROR(E17/907,"")</f>
         <v/>
       </c>
       <c r="G17" s="17">
@@ -1704,7 +1747,7 @@
         <v/>
       </c>
       <c r="H17" s="18">
-        <f>IFERROR(ROUNDUP(G17/D17,0),"")</f>
+        <f>IFERROR(ROUNDUP(G17/907,0),"")</f>
         <v/>
       </c>
       <c r="I17" s="19" t="n"/>
@@ -1719,7 +1762,7 @@
       </c>
       <c r="M17" s="21" t="inlineStr">
         <is>
-          <t>Stay on the 2 lb ($0.44/oz); the 20 oz is $0.48/oz.</t>
+          <t>Stay on the 2 lb ($0.44/oz); the 20 oz is $0.48/oz. Margin Edge shows $0.18/oz — see Flags.</t>
         </is>
       </c>
     </row>
@@ -1739,14 +1782,16 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D18" s="14" t="n">
-        <v>227</v>
+      <c r="D18" s="14" t="inlineStr">
+        <is>
+          <t>227 g</t>
+        </is>
       </c>
       <c r="E18" s="15" t="n">
         <v>21.97</v>
       </c>
       <c r="F18" s="16">
-        <f>IFERROR(E18/D18,"")</f>
+        <f>IFERROR(E18/227,"")</f>
         <v/>
       </c>
       <c r="G18" s="17">
@@ -1754,7 +1799,7 @@
         <v/>
       </c>
       <c r="H18" s="18">
-        <f>IFERROR(ROUNDUP(G18/D18,0),"")</f>
+        <f>IFERROR(ROUNDUP(G18/227,0),"")</f>
         <v/>
       </c>
       <c r="I18" s="19" t="n"/>
@@ -1789,14 +1834,16 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D19" s="14" t="n">
-        <v>96</v>
+      <c r="D19" s="14" t="inlineStr">
+        <is>
+          <t>96 g</t>
+        </is>
       </c>
       <c r="E19" s="15" t="n">
         <v>54.95</v>
       </c>
       <c r="F19" s="16">
-        <f>IFERROR(E19/D19,"")</f>
+        <f>IFERROR(E19/96,"")</f>
         <v/>
       </c>
       <c r="G19" s="17">
@@ -1804,7 +1851,7 @@
         <v/>
       </c>
       <c r="H19" s="18">
-        <f>IFERROR(ROUNDUP(G19/D19,0),"")</f>
+        <f>IFERROR(ROUNDUP(G19/96,0),"")</f>
         <v/>
       </c>
       <c r="I19" s="19" t="n"/>
@@ -1839,14 +1886,16 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D20" s="14" t="n">
-        <v>244</v>
+      <c r="D20" s="14" t="inlineStr">
+        <is>
+          <t>244 g</t>
+        </is>
       </c>
       <c r="E20" s="15" t="n">
         <v>64.17</v>
       </c>
       <c r="F20" s="16">
-        <f>IFERROR(E20/D20,"")</f>
+        <f>IFERROR(E20/244,"")</f>
         <v/>
       </c>
       <c r="G20" s="17">
@@ -1854,7 +1903,7 @@
         <v/>
       </c>
       <c r="H20" s="18">
-        <f>IFERROR(ROUNDUP(G20/D20,0),"")</f>
+        <f>IFERROR(ROUNDUP(G20/244,0),"")</f>
         <v/>
       </c>
       <c r="I20" s="19" t="n"/>
@@ -1869,7 +1918,7 @@
       </c>
       <c r="M20" s="21" t="inlineStr">
         <is>
-          <t>Listing has 4 sizes (6.24/6.63/8.3/8.61 oz). Standardize on 8.61 oz.</t>
+          <t>Listing has 4 sizes. Standardize on 8.61 oz.</t>
         </is>
       </c>
     </row>
@@ -1889,14 +1938,16 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D21" s="14" t="n">
-        <v>425</v>
+      <c r="D21" s="14" t="inlineStr">
+        <is>
+          <t>425 g</t>
+        </is>
       </c>
       <c r="E21" s="15" t="n">
         <v>11.15</v>
       </c>
       <c r="F21" s="16">
-        <f>IFERROR(E21/D21,"")</f>
+        <f>IFERROR(E21/425,"")</f>
         <v/>
       </c>
       <c r="G21" s="17">
@@ -1904,7 +1955,7 @@
         <v/>
       </c>
       <c r="H21" s="18">
-        <f>IFERROR(ROUNDUP(G21/D21,0),"")</f>
+        <f>IFERROR(ROUNDUP(G21/425,0),"")</f>
         <v/>
       </c>
       <c r="I21" s="19" t="n"/>
@@ -1939,14 +1990,16 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D22" s="14" t="n">
-        <v>60</v>
+      <c r="D22" s="14" t="inlineStr">
+        <is>
+          <t>60 g</t>
+        </is>
       </c>
       <c r="E22" s="15" t="n">
         <v>27.26</v>
       </c>
       <c r="F22" s="16">
-        <f>IFERROR(E22/D22,"")</f>
+        <f>IFERROR(E22/60,"")</f>
         <v/>
       </c>
       <c r="G22" s="17">
@@ -1954,7 +2007,7 @@
         <v/>
       </c>
       <c r="H22" s="18">
-        <f>IFERROR(ROUNDUP(G22/D22,0),"")</f>
+        <f>IFERROR(ROUNDUP(G22/60,0),"")</f>
         <v/>
       </c>
       <c r="I22" s="19" t="n"/>
@@ -1989,7 +2042,11 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D23" s="24" t="n"/>
+      <c r="D23" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="E23" s="24" t="n"/>
       <c r="F23" s="24" t="n"/>
       <c r="G23" s="17">
@@ -2003,14 +2060,14 @@
       <c r="L23" s="24" t="n"/>
       <c r="M23" s="22" t="inlineStr">
         <is>
-          <t>Cacao NIBS are cafe-side (acai bowl) and cannot substitute — they won't pass the sift step. Margin Edge has 'Spice, Cocoa Powder' at $1.57/100 g.</t>
+          <t>Cacao NIBS are cafe-side and cannot substitute — they won't pass the sift. Margin Edge has 'Spice, Cocoa Powder' at $1.57/100 g.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="12" t="inlineStr">
         <is>
-          <t>OTHER VENDORS</t>
+          <t>SMOOTHIE POWDER PREP — OTHER VENDORS</t>
         </is>
       </c>
       <c r="B24" s="13" t="n"/>
@@ -2042,14 +2099,16 @@
           <t>Hillcrest</t>
         </is>
       </c>
-      <c r="D25" s="14" t="n">
-        <v>24948</v>
+      <c r="D25" s="14" t="inlineStr">
+        <is>
+          <t>55 lb / 24,948 g</t>
+        </is>
       </c>
       <c r="E25" s="15" t="n">
         <v>214.08</v>
       </c>
       <c r="F25" s="16">
-        <f>IFERROR(E25/D25,"")</f>
+        <f>IFERROR(E25/24948,"")</f>
         <v/>
       </c>
       <c r="G25" s="17">
@@ -2057,7 +2116,7 @@
         <v/>
       </c>
       <c r="H25" s="18">
-        <f>IFERROR(ROUNDUP(G25/D25,0),"")</f>
+        <f>IFERROR(ROUNDUP(G25/24948,0),"")</f>
         <v/>
       </c>
       <c r="I25" s="19" t="n"/>
@@ -2072,7 +2131,7 @@
       </c>
       <c r="M25" s="21" t="inlineStr">
         <is>
-          <t>~14 batches per bag. Bulk drop-ship — confirm lead time, not a 2-day item.</t>
+          <t>~14 batches per bag. Bulk drop-ship — confirm lead time.</t>
         </is>
       </c>
     </row>
@@ -2092,14 +2151,16 @@
           <t>Sante (direct)</t>
         </is>
       </c>
-      <c r="D26" s="14" t="n">
-        <v>250</v>
+      <c r="D26" s="14" t="inlineStr">
+        <is>
+          <t>250 g</t>
+        </is>
       </c>
       <c r="E26" s="15" t="n">
         <v>74.25</v>
       </c>
       <c r="F26" s="16">
-        <f>IFERROR(E26/D26,"")</f>
+        <f>IFERROR(E26/250,"")</f>
         <v/>
       </c>
       <c r="G26" s="17">
@@ -2107,7 +2168,7 @@
         <v/>
       </c>
       <c r="H26" s="18">
-        <f>IFERROR(ROUNDUP(G26/D26,0),"")</f>
+        <f>IFERROR(ROUNDUP(G26/250,0),"")</f>
         <v/>
       </c>
       <c r="I26" s="19" t="n"/>
@@ -2122,14 +2183,14 @@
       </c>
       <c r="M26" s="21" t="inlineStr">
         <is>
-          <t>$74.25/bag net of a 38% account discount (list $120). Sold in 10-bag lots = $742.50, ~46 batches. Order on its own cadence.</t>
+          <t>$74.25/bag net of 38% account discount (list $120). 10-bag lots = $742.50, ~46 batches.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="12" t="inlineStr">
         <is>
-          <t>IN-HOUSE — NOT AN ORDER LINE</t>
+          <t>SMOOTHIE LIQUID MIX — recipes confirmed in Margin Edge, usage not yet mapped</t>
         </is>
       </c>
       <c r="B27" s="13" t="n"/>
@@ -2148,105 +2209,1069 @@
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
+          <t>Coconut Cream</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>Nature's Greatest Organic Coconut Cream, no guar gum</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D28" s="14" t="inlineStr">
+        <is>
+          <t>12 x 13.5 fl oz</t>
+        </is>
+      </c>
+      <c r="E28" s="15" t="n">
+        <v>45.44</v>
+      </c>
+      <c r="F28" s="24" t="n"/>
+      <c r="G28" s="24" t="n"/>
+      <c r="H28" s="24" t="n"/>
+      <c r="I28" s="19" t="n"/>
+      <c r="J28" s="25" t="inlineStr">
+        <is>
+          <t>par</t>
+        </is>
+      </c>
+      <c r="K28" s="19" t="n"/>
+      <c r="L28" s="20">
+        <f>IFERROR(N(K28)*E28,0)</f>
+        <v/>
+      </c>
+      <c r="M28" s="22" t="inlineStr">
+        <is>
+          <t>CONFIRMED: Being Brigid Liquid Mix + Fall Coconut Cream (bar). Margin Edge prices it at $0 — data gap.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Almond Milk</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>Mooala Organic Simple Almond Milk, unsweetened</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D29" s="14" t="inlineStr">
+        <is>
+          <t>6 x 32 oz</t>
+        </is>
+      </c>
+      <c r="E29" s="15" t="n">
+        <v>36.99</v>
+      </c>
+      <c r="F29" s="24" t="n"/>
+      <c r="G29" s="24" t="n"/>
+      <c r="H29" s="24" t="n"/>
+      <c r="I29" s="19" t="n"/>
+      <c r="J29" s="25" t="inlineStr">
+        <is>
+          <t>par</t>
+        </is>
+      </c>
+      <c r="K29" s="19" t="n"/>
+      <c r="L29" s="20">
+        <f>IFERROR(N(K29)*E29,0)</f>
+        <v/>
+      </c>
+      <c r="M29" s="21" t="inlineStr">
+        <is>
+          <t>Liquid Mix component.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Oat Milk Creamer</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>JOI Instant Oat Milk Creamer Pouch</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D30" s="14" t="inlineStr">
+        <is>
+          <t>32 servings</t>
+        </is>
+      </c>
+      <c r="E30" s="15" t="n">
+        <v>30.56</v>
+      </c>
+      <c r="F30" s="24" t="n"/>
+      <c r="G30" s="24" t="n"/>
+      <c r="H30" s="24" t="n"/>
+      <c r="I30" s="19" t="n"/>
+      <c r="J30" s="25" t="inlineStr">
+        <is>
+          <t>par</t>
+        </is>
+      </c>
+      <c r="K30" s="19" t="n"/>
+      <c r="L30" s="20">
+        <f>IFERROR(N(K30)*E30,0)</f>
+        <v/>
+      </c>
+      <c r="M30" s="21" t="inlineStr">
+        <is>
+          <t>Liquid Mix component.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>MCT Oil</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>Nature's Way Organic MCT Oil</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D31" s="14" t="inlineStr">
+        <is>
+          <t>30 fl oz</t>
+        </is>
+      </c>
+      <c r="E31" s="15" t="n">
+        <v>20.17</v>
+      </c>
+      <c r="F31" s="24" t="n"/>
+      <c r="G31" s="24" t="n"/>
+      <c r="H31" s="24" t="n"/>
+      <c r="I31" s="19" t="n"/>
+      <c r="J31" s="25" t="inlineStr">
+        <is>
+          <t>par</t>
+        </is>
+      </c>
+      <c r="K31" s="19" t="n"/>
+      <c r="L31" s="20">
+        <f>IFERROR(N(K31)*E31,0)</f>
+        <v/>
+      </c>
+      <c r="M31" s="21" t="inlineStr">
+        <is>
+          <t>Liquid Mix component.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Beef Protein, Vanilla</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>Equip Foods Prime Protein, Vanilla (grass-fed beef)</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D32" s="14" t="inlineStr">
+        <is>
+          <t>30 servings</t>
+        </is>
+      </c>
+      <c r="E32" s="15" t="n">
+        <v>64.63</v>
+      </c>
+      <c r="F32" s="24" t="n"/>
+      <c r="G32" s="24" t="n"/>
+      <c r="H32" s="24" t="n"/>
+      <c r="I32" s="19" t="n"/>
+      <c r="J32" s="25" t="inlineStr">
+        <is>
+          <t>par</t>
+        </is>
+      </c>
+      <c r="K32" s="19" t="n"/>
+      <c r="L32" s="20">
+        <f>IFERROR(N(K32)*E32,0)</f>
+        <v/>
+      </c>
+      <c r="M32" s="21" t="inlineStr">
+        <is>
+          <t>Liquid Mix component.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Cashew Butter</t>
+        </is>
+      </c>
+      <c r="B33" s="23" t="inlineStr">
+        <is>
+          <t>** NO SKU CONFIRMED **</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D33" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E33" s="24" t="n"/>
+      <c r="F33" s="24" t="n"/>
+      <c r="G33" s="24" t="n"/>
+      <c r="H33" s="24" t="n"/>
+      <c r="I33" s="24" t="n"/>
+      <c r="J33" s="24" t="n"/>
+      <c r="K33" s="24" t="n"/>
+      <c r="L33" s="24" t="n"/>
+      <c r="M33" s="22" t="inlineStr">
+        <is>
+          <t>Being Brigid Liquid Mix uses 330 g. Margin Edge prices it at $8.53 — need the purchased SKU.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="12" t="inlineStr">
+        <is>
+          <t>COCKTAIL / BAR PREP</t>
+        </is>
+      </c>
+      <c r="B34" s="13" t="n"/>
+      <c r="C34" s="13" t="n"/>
+      <c r="D34" s="13" t="n"/>
+      <c r="E34" s="13" t="n"/>
+      <c r="F34" s="13" t="n"/>
+      <c r="G34" s="13" t="n"/>
+      <c r="H34" s="13" t="n"/>
+      <c r="I34" s="13" t="n"/>
+      <c r="J34" s="13" t="n"/>
+      <c r="K34" s="13" t="n"/>
+      <c r="L34" s="13" t="n"/>
+      <c r="M34" s="13" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Chai, Loose Leaf</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>Davidson's Tea Bulk, Classic Chai</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D35" s="14" t="inlineStr">
+        <is>
+          <t>16 oz</t>
+        </is>
+      </c>
+      <c r="E35" s="15" t="n">
+        <v>19.12</v>
+      </c>
+      <c r="F35" s="24" t="n"/>
+      <c r="G35" s="24" t="n"/>
+      <c r="H35" s="24" t="n"/>
+      <c r="I35" s="19" t="n"/>
+      <c r="J35" s="25" t="inlineStr">
+        <is>
+          <t>par</t>
+        </is>
+      </c>
+      <c r="K35" s="19" t="n"/>
+      <c r="L35" s="20">
+        <f>IFERROR(N(K35)*E35,0)</f>
+        <v/>
+      </c>
+      <c r="M35" s="22" t="inlineStr">
+        <is>
+          <t>CONFIRMED: 'Brewed Chai Tea' bar prep (4 fl oz per 32 oz batch). Margin Edge prices it at $0 — data gap.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Chai Concentrate</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>Bhakti Chai Tea Concentrate, Unsweetened</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D36" s="14" t="inlineStr">
+        <is>
+          <t>2-pack, 16 srv</t>
+        </is>
+      </c>
+      <c r="E36" s="15" t="n">
+        <v>19.99</v>
+      </c>
+      <c r="F36" s="24" t="n"/>
+      <c r="G36" s="24" t="n"/>
+      <c r="H36" s="24" t="n"/>
+      <c r="I36" s="19" t="n"/>
+      <c r="J36" s="25" t="inlineStr">
+        <is>
+          <t>par</t>
+        </is>
+      </c>
+      <c r="K36" s="19" t="n"/>
+      <c r="L36" s="20">
+        <f>IFERROR(N(K36)*E36,0)</f>
+        <v/>
+      </c>
+      <c r="M36" s="21" t="inlineStr">
+        <is>
+          <t>Second chai format. Confirm both are needed — concentrate vs loose leaf.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Hibiscus Flowers</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>Organic Hibiscus Flowers, cut &amp; sifted</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D37" s="14" t="inlineStr">
+        <is>
+          <t>2 lb</t>
+        </is>
+      </c>
+      <c r="E37" s="15" t="n">
+        <v>27.51</v>
+      </c>
+      <c r="F37" s="24" t="n"/>
+      <c r="G37" s="24" t="n"/>
+      <c r="H37" s="24" t="n"/>
+      <c r="I37" s="19" t="n"/>
+      <c r="J37" s="25" t="inlineStr">
+        <is>
+          <t>par</t>
+        </is>
+      </c>
+      <c r="K37" s="19" t="n"/>
+      <c r="L37" s="20">
+        <f>IFERROR(N(K37)*E37,0)</f>
+        <v/>
+      </c>
+      <c r="M37" s="21" t="inlineStr">
+        <is>
+          <t>Feeds Hibiscus Cinnamon Simple, Hibiscus Limeade Bulk, Hibiscus Allulose Syrup.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Agave Syrup</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>Blue Green Organics Raw Blue Agave Syrup</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D38" s="14" t="inlineStr">
+        <is>
+          <t>176 oz</t>
+        </is>
+      </c>
+      <c r="E38" s="15" t="n">
+        <v>45.59</v>
+      </c>
+      <c r="F38" s="24" t="n"/>
+      <c r="G38" s="24" t="n"/>
+      <c r="H38" s="24" t="n"/>
+      <c r="I38" s="19" t="n"/>
+      <c r="J38" s="25" t="inlineStr">
+        <is>
+          <t>par</t>
+        </is>
+      </c>
+      <c r="K38" s="19" t="n"/>
+      <c r="L38" s="20">
+        <f>IFERROR(N(K38)*E38,0)</f>
+        <v/>
+      </c>
+      <c r="M38" s="21" t="inlineStr">
+        <is>
+          <t>Bulk sweetener. Qty 2 last ordered.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Vanilla Bean Paste</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>Simply Organic Vanilla Bean Paste</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D39" s="14" t="inlineStr">
+        <is>
+          <t>4 oz jar</t>
+        </is>
+      </c>
+      <c r="E39" s="15" t="n">
+        <v>17.89</v>
+      </c>
+      <c r="F39" s="24" t="n"/>
+      <c r="G39" s="24" t="n"/>
+      <c r="H39" s="24" t="n"/>
+      <c r="I39" s="19" t="n"/>
+      <c r="J39" s="25" t="inlineStr">
+        <is>
+          <t>par</t>
+        </is>
+      </c>
+      <c r="K39" s="19" t="n"/>
+      <c r="L39" s="20">
+        <f>IFERROR(N(K39)*E39,0)</f>
+        <v/>
+      </c>
+      <c r="M39" s="21" t="inlineStr">
+        <is>
+          <t>Qty 10 last ordered — high volume for 4 oz jars. Check if a larger pack exists.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Star Anise, Whole</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>Frontier Co-op Organic Whole Star Anise</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D40" s="14" t="inlineStr">
+        <is>
+          <t>1 lb</t>
+        </is>
+      </c>
+      <c r="E40" s="15" t="n">
+        <v>33.52</v>
+      </c>
+      <c r="F40" s="24" t="n"/>
+      <c r="G40" s="24" t="n"/>
+      <c r="H40" s="24" t="n"/>
+      <c r="I40" s="19" t="n"/>
+      <c r="J40" s="25" t="inlineStr">
+        <is>
+          <t>par</t>
+        </is>
+      </c>
+      <c r="K40" s="19" t="n"/>
+      <c r="L40" s="20">
+        <f>IFERROR(N(K40)*E40,0)</f>
+        <v/>
+      </c>
+      <c r="M40" s="21" t="inlineStr">
+        <is>
+          <t>Qty 4 last ordered.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Pumpkin Pie Spice</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>Frontier Organic Pumpkin Pie Spice</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D41" s="14" t="inlineStr">
+        <is>
+          <t>16 oz</t>
+        </is>
+      </c>
+      <c r="E41" s="15" t="n">
+        <v>13.12</v>
+      </c>
+      <c r="F41" s="24" t="n"/>
+      <c r="G41" s="24" t="n"/>
+      <c r="H41" s="24" t="n"/>
+      <c r="I41" s="19" t="n"/>
+      <c r="J41" s="25" t="inlineStr">
+        <is>
+          <t>par</t>
+        </is>
+      </c>
+      <c r="K41" s="19" t="n"/>
+      <c r="L41" s="20">
+        <f>IFERROR(N(K41)*E41,0)</f>
+        <v/>
+      </c>
+      <c r="M41" s="21" t="inlineStr">
+        <is>
+          <t>Seasonal. NOT a cinnamon substitute — it's a blend.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Pecans, Raw</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>Yupik Organic Raw Pecans, unsalted</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D42" s="14" t="inlineStr">
+        <is>
+          <t>2.2 lb</t>
+        </is>
+      </c>
+      <c r="E42" s="15" t="n">
+        <v>39.93</v>
+      </c>
+      <c r="F42" s="24" t="n"/>
+      <c r="G42" s="24" t="n"/>
+      <c r="H42" s="24" t="n"/>
+      <c r="I42" s="19" t="n"/>
+      <c r="J42" s="25" t="inlineStr">
+        <is>
+          <t>par</t>
+        </is>
+      </c>
+      <c r="K42" s="19" t="n"/>
+      <c r="L42" s="20">
+        <f>IFERROR(N(K42)*E42,0)</f>
+        <v/>
+      </c>
+      <c r="M42" s="21" t="inlineStr">
+        <is>
+          <t>Qty 2-4 per order.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Coconut Sugar</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>MADHAVA Organic Coconut Sugar</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D43" s="14" t="inlineStr">
+        <is>
+          <t>6 x 1 lb</t>
+        </is>
+      </c>
+      <c r="E43" s="15" t="n">
+        <v>14.26</v>
+      </c>
+      <c r="F43" s="24" t="n"/>
+      <c r="G43" s="24" t="n"/>
+      <c r="H43" s="24" t="n"/>
+      <c r="I43" s="19" t="n"/>
+      <c r="J43" s="25" t="inlineStr">
+        <is>
+          <t>par</t>
+        </is>
+      </c>
+      <c r="K43" s="19" t="n"/>
+      <c r="L43" s="20">
+        <f>IFERROR(N(K43)*E43,0)</f>
+        <v/>
+      </c>
+      <c r="M43" s="22" t="inlineStr">
+        <is>
+          <t>Verify whether $14.26 is the 6-pack or per bag — unusually low for a 6-pack.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Graham Crackers</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>Annie's Organic Honey Graham Crackers</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D44" s="14" t="inlineStr">
+        <is>
+          <t>14.4 oz</t>
+        </is>
+      </c>
+      <c r="E44" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="F44" s="24" t="n"/>
+      <c r="G44" s="24" t="n"/>
+      <c r="H44" s="24" t="n"/>
+      <c r="I44" s="19" t="n"/>
+      <c r="J44" s="25" t="inlineStr">
+        <is>
+          <t>par</t>
+        </is>
+      </c>
+      <c r="K44" s="19" t="n"/>
+      <c r="L44" s="20">
+        <f>IFERROR(N(K44)*E44,0)</f>
+        <v/>
+      </c>
+      <c r="M44" s="21" t="inlineStr">
+        <is>
+          <t>Rim / garnish. Confirm which drink or dessert.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="12" t="inlineStr">
+        <is>
+          <t>CAFE</t>
+        </is>
+      </c>
+      <c r="B45" s="13" t="n"/>
+      <c r="C45" s="13" t="n"/>
+      <c r="D45" s="13" t="n"/>
+      <c r="E45" s="13" t="n"/>
+      <c r="F45" s="13" t="n"/>
+      <c r="G45" s="13" t="n"/>
+      <c r="H45" s="13" t="n"/>
+      <c r="I45" s="13" t="n"/>
+      <c r="J45" s="13" t="n"/>
+      <c r="K45" s="13" t="n"/>
+      <c r="L45" s="13" t="n"/>
+      <c r="M45" s="13" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>Cacao Nibs</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>Anthony's Organic Cacao Cocoa Nibs, Criollo, 2 lb</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D46" s="14" t="inlineStr">
+        <is>
+          <t>907 g</t>
+        </is>
+      </c>
+      <c r="E46" s="15" t="n">
+        <v>34.99</v>
+      </c>
+      <c r="F46" s="16">
+        <f>IFERROR(E46/907,"")</f>
+        <v/>
+      </c>
+      <c r="G46" s="24" t="n"/>
+      <c r="H46" s="24" t="n"/>
+      <c r="I46" s="19" t="n"/>
+      <c r="J46" s="25" t="inlineStr">
+        <is>
+          <t>par</t>
+        </is>
+      </c>
+      <c r="K46" s="19" t="n"/>
+      <c r="L46" s="20">
+        <f>IFERROR(N(K46)*E46,0)</f>
+        <v/>
+      </c>
+      <c r="M46" s="21" t="inlineStr">
+        <is>
+          <t>Acai bowl. Cheaper per gram than Viva ($0.0386 vs $0.0427).</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Cacao Nibs (alt)</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>Viva Naturals Organic Cacao Nibs, unsweetened, 1 lb</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D47" s="14" t="inlineStr">
+        <is>
+          <t>454 g</t>
+        </is>
+      </c>
+      <c r="E47" s="15" t="n">
+        <v>19.39</v>
+      </c>
+      <c r="F47" s="16">
+        <f>IFERROR(E47/454,"")</f>
+        <v/>
+      </c>
+      <c r="G47" s="24" t="n"/>
+      <c r="H47" s="24" t="n"/>
+      <c r="I47" s="19" t="n"/>
+      <c r="J47" s="25" t="inlineStr">
+        <is>
+          <t>par</t>
+        </is>
+      </c>
+      <c r="K47" s="19" t="n"/>
+      <c r="L47" s="20">
+        <f>IFERROR(N(K47)*E47,0)</f>
+        <v/>
+      </c>
+      <c r="M47" s="21" t="inlineStr">
+        <is>
+          <t>Acai bowl. Second nib SKU — confirm both are needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="12" t="inlineStr">
+        <is>
+          <t>UNASSIGNED — bought, but not tied to a recipe. Do not order until confirmed.</t>
+        </is>
+      </c>
+      <c r="B48" s="13" t="n"/>
+      <c r="C48" s="13" t="n"/>
+      <c r="D48" s="13" t="n"/>
+      <c r="E48" s="13" t="n"/>
+      <c r="F48" s="13" t="n"/>
+      <c r="G48" s="13" t="n"/>
+      <c r="H48" s="13" t="n"/>
+      <c r="I48" s="13" t="n"/>
+      <c r="J48" s="13" t="n"/>
+      <c r="K48" s="13" t="n"/>
+      <c r="L48" s="13" t="n"/>
+      <c r="M48" s="13" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>Peanut Butter Powder (sweetened)</t>
+        </is>
+      </c>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>Lakanto Peanut Butter Powder, monk-fruit sweetened</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D49" s="14" t="inlineStr">
+        <is>
+          <t>8.5 oz</t>
+        </is>
+      </c>
+      <c r="E49" s="15" t="n">
+        <v>13.36</v>
+      </c>
+      <c r="F49" s="24" t="n"/>
+      <c r="G49" s="24" t="n"/>
+      <c r="H49" s="24" t="n"/>
+      <c r="I49" s="19" t="n"/>
+      <c r="J49" s="25" t="inlineStr">
+        <is>
+          <t>par</t>
+        </is>
+      </c>
+      <c r="K49" s="19" t="n"/>
+      <c r="L49" s="20">
+        <f>IFERROR(N(K49)*E49,0)</f>
+        <v/>
+      </c>
+      <c r="M49" s="22" t="inlineStr">
+        <is>
+          <t>NOT the smoothie PB powder. Store apart from prep stock to avoid a mix-up.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Collagen Peptides, Unflavored</t>
+        </is>
+      </c>
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t>Orgain Hydrolyzed Collagen Peptides, Unflavored, 1 lb</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D50" s="14" t="inlineStr">
+        <is>
+          <t>454 g</t>
+        </is>
+      </c>
+      <c r="E50" s="15" t="n">
+        <v>21.12</v>
+      </c>
+      <c r="F50" s="24" t="n"/>
+      <c r="G50" s="24" t="n"/>
+      <c r="H50" s="24" t="n"/>
+      <c r="I50" s="19" t="n"/>
+      <c r="J50" s="25" t="inlineStr">
+        <is>
+          <t>par</t>
+        </is>
+      </c>
+      <c r="K50" s="19" t="n"/>
+      <c r="L50" s="20">
+        <f>IFERROR(N(K50)*E50,0)</f>
+        <v/>
+      </c>
+      <c r="M50" s="22" t="inlineStr">
+        <is>
+          <t>Bought 9/21/2026 but appears in no powder prep recipe. Identify the use.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="12" t="inlineStr">
+        <is>
+          <t>IN-HOUSE — NOT AN ORDER LINE</t>
+        </is>
+      </c>
+      <c r="B51" s="13" t="n"/>
+      <c r="C51" s="13" t="n"/>
+      <c r="D51" s="13" t="n"/>
+      <c r="E51" s="13" t="n"/>
+      <c r="F51" s="13" t="n"/>
+      <c r="G51" s="13" t="n"/>
+      <c r="H51" s="13" t="n"/>
+      <c r="I51" s="13" t="n"/>
+      <c r="J51" s="13" t="n"/>
+      <c r="K51" s="13" t="n"/>
+      <c r="L51" s="13" t="n"/>
+      <c r="M51" s="13" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
           <t>Cinnamon, Ground</t>
         </is>
       </c>
-      <c r="B28" s="4" t="inlineStr">
+      <c r="B52" s="4" t="inlineStr">
         <is>
           <t>Carried in kitchen stock</t>
         </is>
       </c>
-      <c r="C28" s="4" t="inlineStr">
+      <c r="C52" s="4" t="inlineStr">
         <is>
           <t>In-house</t>
         </is>
       </c>
-      <c r="D28" s="24" t="n"/>
-      <c r="E28" s="24" t="n"/>
-      <c r="F28" s="24" t="n"/>
-      <c r="G28" s="17">
+      <c r="D52" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E52" s="24" t="n"/>
+      <c r="F52" s="24" t="n"/>
+      <c r="G52" s="17">
         <f>'Recipe Usage'!F24</f>
         <v/>
       </c>
-      <c r="H28" s="24" t="n"/>
-      <c r="I28" s="24" t="n"/>
-      <c r="J28" s="24" t="n"/>
-      <c r="K28" s="24" t="n"/>
-      <c r="L28" s="24" t="n"/>
-      <c r="M28" s="21" t="inlineStr">
+      <c r="H52" s="24" t="n"/>
+      <c r="I52" s="24" t="n"/>
+      <c r="J52" s="24" t="n"/>
+      <c r="K52" s="24" t="n"/>
+      <c r="L52" s="24" t="n"/>
+      <c r="M52" s="21" t="inlineStr">
         <is>
           <t>Pull from stock. Stays on the prep guide, excluded from ordering.</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="25" t="inlineStr">
+    <row r="53">
+      <c r="A53" s="26" t="inlineStr">
         <is>
           <t>ORDER TOTAL (this location)</t>
         </is>
       </c>
-      <c r="B29" s="26" t="n"/>
-      <c r="C29" s="26" t="n"/>
-      <c r="D29" s="26" t="n"/>
-      <c r="E29" s="26" t="n"/>
-      <c r="F29" s="26" t="n"/>
-      <c r="G29" s="26" t="n"/>
-      <c r="H29" s="26" t="n"/>
-      <c r="I29" s="26" t="n"/>
-      <c r="J29" s="26" t="n"/>
-      <c r="K29" s="26" t="n"/>
-      <c r="L29" s="27">
-        <f>SUM(L6:L28)</f>
-        <v/>
-      </c>
-      <c r="M29" s="26" t="n"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="28" t="inlineStr">
+      <c r="B53" s="27" t="n"/>
+      <c r="C53" s="27" t="n"/>
+      <c r="D53" s="27" t="n"/>
+      <c r="E53" s="27" t="n"/>
+      <c r="F53" s="27" t="n"/>
+      <c r="G53" s="27" t="n"/>
+      <c r="H53" s="27" t="n"/>
+      <c r="I53" s="27" t="n"/>
+      <c r="J53" s="27" t="n"/>
+      <c r="K53" s="27" t="n"/>
+      <c r="L53" s="28">
+        <f>SUM(L6:L52)</f>
+        <v/>
+      </c>
+      <c r="M53" s="27" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="29" t="inlineStr">
         <is>
           <t>LEGEND</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="29" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="30" t="inlineStr">
         <is>
           <t>Yellow cells = you fill in (On Hand, Order Qty)</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="30" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="31" t="inlineStr">
         <is>
           <t>Blue text = fixed data (pack size, price). Update when prices change.</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="31" t="inlineStr">
+    <row r="58">
+      <c r="A58" s="32" t="inlineStr">
         <is>
           <t>Green text = pulled from the 'Recipe Usage' tab</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="32" t="inlineStr">
+    <row r="59">
+      <c r="A59" s="30" t="inlineStr">
         <is>
           <t>Black text = calculated — do not overwrite</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="33" t="inlineStr">
+    <row r="60">
+      <c r="A60" s="33" t="inlineStr">
         <is>
           <t>Red text = needs a decision. See the 'Notes &amp; Flags' tab.</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>EXAMPLE: if Chia shows 3 packs/cycle and you have 1 on hand, Suggested = 2. Enter 2 (or your own number) in Order Qty.</t>
+    <row r="61">
+      <c r="A61" s="34" t="inlineStr">
+        <is>
+          <t>"par" in Suggested = no recipe usage mapped yet; order to par by eye until the recipe lands.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Chia shows 3 packs/cycle. Enter 1 in On Hand, Suggested reads 2. Enter 2 in Order Qty and Ext. Cost reads $27.94.</t>
         </is>
       </c>
     </row>
@@ -2261,14 +3286,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="54" customWidth="1" min="3" max="3"/>
+    <col width="56" customWidth="1" min="3" max="3"/>
     <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="50" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2279,304 +3304,429 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="34" t="inlineStr">
+      <c r="A3" s="35" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B3" s="34" t="inlineStr">
+      <c r="B3" s="35" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="C3" s="34" t="inlineStr">
+      <c r="C3" s="35" t="inlineStr">
         <is>
           <t>Issue</t>
         </is>
       </c>
-      <c r="D3" s="34" t="inlineStr">
+      <c r="D3" s="35" t="inlineStr">
         <is>
           <t>Impact</t>
         </is>
       </c>
-      <c r="E3" s="34" t="inlineStr">
+      <c r="E3" s="35" t="inlineStr">
         <is>
           <t>What's needed</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="46" customHeight="1">
-      <c r="A4" s="35" t="n">
+    <row r="4" ht="48" customHeight="1">
+      <c r="A4" s="36" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="36" t="inlineStr">
+      <c r="B4" s="37" t="inlineStr">
         <is>
           <t>Cocoa Powder</t>
         </is>
       </c>
-      <c r="C4" s="37" t="inlineStr">
+      <c r="C4" s="38" t="inlineStr">
         <is>
           <t>Keto calls for 100 g cocoa powder. No SKU confirmed. Cacao nibs in order history are cafe-side (acai bowl) and won't pass the fine-mesh sift.</t>
         </is>
       </c>
-      <c r="D4" s="37" t="inlineStr">
+      <c r="D4" s="38" t="inlineStr">
         <is>
           <t>Keto batch cannot be fully costed or ordered.</t>
         </is>
       </c>
-      <c r="E4" s="37" t="inlineStr">
+      <c r="E4" s="38" t="inlineStr">
         <is>
           <t>Confirm a milled cocoa powder SKU. Margin Edge has 'Spice, Cocoa Powder' at $1.57/100 g.</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="46" customHeight="1">
-      <c r="A5" s="35" t="n">
+    <row r="5" ht="48" customHeight="1">
+      <c r="A5" s="36" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="36" t="inlineStr">
+      <c r="B5" s="37" t="inlineStr">
         <is>
           <t>Bovine Colostrum</t>
         </is>
       </c>
-      <c r="C5" s="37" t="inlineStr">
+      <c r="C5" s="38" t="inlineStr">
         <is>
           <t>Recipe 100 g vs 96 g jar — 4 g (4.2%) over forces a second jar and strands 92 g.</t>
         </is>
       </c>
-      <c r="D5" s="37" t="inlineStr">
+      <c r="D5" s="38" t="inlineStr">
         <is>
           <t>$54.95 per Longevity batch.</t>
         </is>
       </c>
-      <c r="E5" s="37" t="inlineStr">
+      <c r="E5" s="38" t="inlineStr">
         <is>
           <t>Decide: round the recipe to 96 g, or keep 100 g and accept 2 jars.</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="46" customHeight="1">
-      <c r="A6" s="35" t="n">
+    <row r="6" ht="48" customHeight="1">
+      <c r="A6" s="36" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="36" t="inlineStr">
+      <c r="B6" s="37" t="inlineStr">
         <is>
           <t>Peanut Butter Powder</t>
         </is>
       </c>
-      <c r="C6" s="37" t="inlineStr">
+      <c r="C6" s="38" t="inlineStr">
         <is>
           <t>Recipe 1,875 g vs 1,814 g bag — 61 g (3.4%) over forces a second bag.</t>
         </is>
       </c>
-      <c r="D6" s="37" t="inlineStr">
+      <c r="D6" s="38" t="inlineStr">
         <is>
           <t>$28.41 per Keto batch, plus 1,753 g idle.</t>
         </is>
       </c>
-      <c r="E6" s="37" t="inlineStr">
+      <c r="E6" s="38" t="inlineStr">
         <is>
           <t>Decide: round to 1,814 g (one clean bag) or keep 1,875 g.</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="46" customHeight="1">
-      <c r="A7" s="35" t="n">
+    <row r="7" ht="48" customHeight="1">
+      <c r="A7" s="36" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="36" t="inlineStr">
+      <c r="B7" s="37" t="inlineStr">
         <is>
           <t>Flax Seed</t>
         </is>
       </c>
-      <c r="C7" s="37" t="inlineStr">
+      <c r="C7" s="38" t="inlineStr">
         <is>
           <t>Slide says 35 g; Margin Edge says 135 g.</t>
         </is>
       </c>
-      <c r="D7" s="37" t="inlineStr">
+      <c r="D7" s="38" t="inlineStr">
         <is>
           <t>Being Brigid batch weight and cost.</t>
         </is>
       </c>
-      <c r="E7" s="37" t="inlineStr">
+      <c r="E7" s="38" t="inlineStr">
         <is>
           <t>Confirm the correct quantity. This guide uses 35 g.</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="46" customHeight="1">
-      <c r="A8" s="35" t="n">
+    <row r="8" ht="48" customHeight="1">
+      <c r="A8" s="36" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="36" t="inlineStr">
+      <c r="B8" s="37" t="inlineStr">
         <is>
           <t>BHB Ketones</t>
         </is>
       </c>
-      <c r="C8" s="37" t="inlineStr">
+      <c r="C8" s="38" t="inlineStr">
         <is>
           <t>Slide says Base Ketones; Margin Edge uses Perfect Keto NOOTROPIC Brain Support.</t>
         </is>
       </c>
-      <c r="D8" s="37" t="inlineStr">
+      <c r="D8" s="38" t="inlineStr">
         <is>
           <t>Different product at similar price.</t>
         </is>
       </c>
-      <c r="E8" s="37" t="inlineStr">
+      <c r="E8" s="38" t="inlineStr">
         <is>
           <t>Confirm which product Keto actually uses.</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="46" customHeight="1">
-      <c r="A9" s="35" t="n">
+    <row r="9" ht="48" customHeight="1">
+      <c r="A9" s="36" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="36" t="inlineStr">
+      <c r="B9" s="37" t="inlineStr">
         <is>
           <t>Creatine</t>
         </is>
       </c>
-      <c r="C9" s="37" t="inlineStr">
+      <c r="C9" s="38" t="inlineStr">
         <is>
           <t>Slides say "liposomal creatine"; the product is micronized creatine MONOHYDRATE.</t>
         </is>
       </c>
-      <c r="D9" s="37" t="inlineStr">
+      <c r="D9" s="38" t="inlineStr">
         <is>
           <t>Wording only, if monohydrate is intended.</t>
         </is>
       </c>
-      <c r="E9" s="37" t="inlineStr">
+      <c r="E9" s="38" t="inlineStr">
         <is>
           <t>Reword the slides, or source an actual liposomal product.</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="46" customHeight="1">
-      <c r="A10" s="35" t="n">
+    <row r="10" ht="48" customHeight="1">
+      <c r="A10" s="36" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="36" t="inlineStr">
+      <c r="B10" s="37" t="inlineStr">
         <is>
           <t>Matcha</t>
         </is>
       </c>
-      <c r="C10" s="37" t="inlineStr">
+      <c r="C10" s="38" t="inlineStr">
         <is>
           <t>This guide uses Sante Ceremonial at $0.297/g. Margin Edge uses a generic matcha at $0.047/g.</t>
         </is>
       </c>
-      <c r="D10" s="37" t="inlineStr">
+      <c r="D10" s="38" t="inlineStr">
         <is>
           <t>~$13.50 per Being Brigid batch; 6x price difference.</t>
         </is>
       </c>
-      <c r="E10" s="37" t="inlineStr">
+      <c r="E10" s="38" t="inlineStr">
         <is>
           <t>Confirm whether Being Brigid uses Sante or the generic.</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="46" customHeight="1">
-      <c r="A11" s="35" t="n">
+    <row r="11" ht="48" customHeight="1">
+      <c r="A11" s="36" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="36" t="inlineStr">
+      <c r="B11" s="37" t="inlineStr">
         <is>
           <t>Chocolate Collagen</t>
         </is>
       </c>
-      <c r="C11" s="37" t="inlineStr">
-        <is>
-          <t>Amazon Orgain is a 400 g pack at $2.00/oz. Margin Edge carries a 19.3 oz pack: $2.94/oz at Columbus, $1.40/oz at Cleveland.</t>
-        </is>
-      </c>
-      <c r="D11" s="37" t="inlineStr">
+      <c r="C11" s="38" t="inlineStr">
+        <is>
+          <t>Amazon Orgain is a 400 g pack at $2.00/oz. Margin Edge carries a 19.3 oz pack: $2.94/oz Columbus, $1.40/oz Cleveland.</t>
+        </is>
+      </c>
+      <c r="D11" s="38" t="inlineStr">
         <is>
           <t>Up to $163 per Longevity batch between locations.</t>
         </is>
       </c>
-      <c r="E11" s="37" t="inlineStr">
-        <is>
-          <t>Confirm which pack is actually bought, and why Columbus pays 2.1x Cleveland.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="46" customHeight="1">
-      <c r="A12" s="35" t="n">
+      <c r="E11" s="38" t="inlineStr">
+        <is>
+          <t>Confirm which pack is bought, and why Columbus pays 2.1x Cleveland.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="48" customHeight="1">
+      <c r="A12" s="36" t="n">
         <v>9</v>
       </c>
-      <c r="B12" s="36" t="inlineStr">
+      <c r="B12" s="37" t="inlineStr">
         <is>
           <t>Chia Seeds</t>
         </is>
       </c>
-      <c r="C12" s="37" t="inlineStr">
+      <c r="C12" s="38" t="inlineStr">
         <is>
           <t>Amazon is $0.44/oz. Margin Edge shows $0.18/oz, bought regularly through 9/8/2026.</t>
         </is>
       </c>
-      <c r="D12" s="37" t="inlineStr">
+      <c r="D12" s="38" t="inlineStr">
         <is>
           <t>This guide may overstate chia by ~2.4x.</t>
         </is>
       </c>
-      <c r="E12" s="37" t="inlineStr">
+      <c r="E12" s="38" t="inlineStr">
         <is>
           <t>Confirm whether chia comes from Amazon or a foodservice vendor.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="46" customHeight="1">
-      <c r="A13" s="35" t="n">
+    <row r="13" ht="48" customHeight="1">
+      <c r="A13" s="36" t="n">
         <v>10</v>
       </c>
-      <c r="B13" s="36" t="inlineStr">
+      <c r="B13" s="37" t="inlineStr">
         <is>
           <t>Two locations</t>
         </is>
       </c>
-      <c r="C13" s="37" t="inlineStr">
+      <c r="C13" s="38" t="inlineStr">
         <is>
           <t>Columbus and Cleveland both run this prep. This sheet is ONE location.</t>
         </is>
       </c>
-      <c r="D13" s="37" t="inlineStr">
+      <c r="D13" s="38" t="inlineStr">
         <is>
           <t>Doubling gives ~2x cost, but several packs carry 10-46 batches of runway.</t>
         </is>
       </c>
-      <c r="E13" s="37" t="inlineStr">
-        <is>
-          <t>Decide split vs duplicate: order per site for fast movers; order once and split for 4+ batch runway items.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="46" customHeight="1">
-      <c r="A14" s="35" t="n">
+      <c r="E13" s="38" t="inlineStr">
+        <is>
+          <t>Decide split vs duplicate: per site for fast movers, order once and split for 4+ batch runway.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="48" customHeight="1">
+      <c r="A14" s="36" t="n">
         <v>11</v>
       </c>
-      <c r="B14" s="36" t="inlineStr">
+      <c r="B14" s="37" t="inlineStr">
         <is>
           <t>Batch frequency</t>
         </is>
       </c>
-      <c r="C14" s="37" t="inlineStr">
+      <c r="C14" s="38" t="inlineStr">
         <is>
           <t>Unknown.</t>
         </is>
       </c>
-      <c r="D14" s="37" t="inlineStr">
+      <c r="D14" s="38" t="inlineStr">
         <is>
           <t>Cannot convert per-cycle quantities into a reorder cadence or par levels.</t>
         </is>
       </c>
-      <c r="E14" s="37" t="inlineStr">
+      <c r="E14" s="38" t="inlineStr">
         <is>
           <t>Provide how often each batch is run, per location.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="48" customHeight="1">
+      <c r="A15" s="36" t="n">
+        <v>12</v>
+      </c>
+      <c r="B15" s="37" t="inlineStr">
+        <is>
+          <t>Cocktail usage</t>
+        </is>
+      </c>
+      <c r="C15" s="38" t="inlineStr">
+        <is>
+          <t>Cocktail, cafe and liquid-mix lines have no grams-per-cycle mapped, so they show "par" instead of a suggested qty.</t>
+        </is>
+      </c>
+      <c r="D15" s="38" t="inlineStr">
+        <is>
+          <t>Those lines must be ordered by eye until mapped.</t>
+        </is>
+      </c>
+      <c r="E15" s="38" t="inlineStr">
+        <is>
+          <t>Margin Edge has 23 'TH - Bar Prep' recipes (see Bar Prep Reference tab). Map products to them to make these lines calculate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="48" customHeight="1">
+      <c r="A16" s="36" t="n">
+        <v>13</v>
+      </c>
+      <c r="B16" s="37" t="inlineStr">
+        <is>
+          <t>Zero-cost products</t>
+        </is>
+      </c>
+      <c r="C16" s="38" t="inlineStr">
+        <is>
+          <t>Margin Edge prices Coconut Cream, Loose Leaf Chai and Sea Moss at $0.00 in some recipes.</t>
+        </is>
+      </c>
+      <c r="D16" s="38" t="inlineStr">
+        <is>
+          <t>Bar and liquid-mix recipe costs are understated.</t>
+        </is>
+      </c>
+      <c r="E16" s="38" t="inlineStr">
+        <is>
+          <t>Add real costs to those products in Margin Edge.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="48" customHeight="1">
+      <c r="A17" s="36" t="n">
+        <v>14</v>
+      </c>
+      <c r="B17" s="37" t="inlineStr">
+        <is>
+          <t>Water costed at Columbus</t>
+        </is>
+      </c>
+      <c r="C17" s="38" t="inlineStr">
+        <is>
+          <t>Margin Edge charges $42.20 for 110 fl oz of water in Being Brigid Liquid Mix and $12.28 for 32 fl oz in Brewed Chai Tea. Cleveland charges $0.00.</t>
+        </is>
+      </c>
+      <c r="D17" s="38" t="inlineStr">
+        <is>
+          <t>Inflates every Columbus recipe that includes water.</t>
+        </is>
+      </c>
+      <c r="E17" s="38" t="inlineStr">
+        <is>
+          <t>Zero out the water product cost at Columbus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="48" customHeight="1">
+      <c r="A18" s="36" t="n">
+        <v>15</v>
+      </c>
+      <c r="B18" s="37" t="inlineStr">
+        <is>
+          <t>Vanilla Bean Paste</t>
+        </is>
+      </c>
+      <c r="C18" s="38" t="inlineStr">
+        <is>
+          <t>Qty 10 of a 4 oz jar per order at $17.89 each = $178.90.</t>
+        </is>
+      </c>
+      <c r="D18" s="38" t="inlineStr">
+        <is>
+          <t>High spend on a small pack format.</t>
+        </is>
+      </c>
+      <c r="E18" s="38" t="inlineStr">
+        <is>
+          <t>Check whether a larger pack or a food-service vanilla exists.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="48" customHeight="1">
+      <c r="A19" s="36" t="n">
+        <v>16</v>
+      </c>
+      <c r="B19" s="37" t="inlineStr">
+        <is>
+          <t>Coconut Sugar</t>
+        </is>
+      </c>
+      <c r="C19" s="38" t="inlineStr">
+        <is>
+          <t>$14.26 listed for a 6 x 1 lb pack is unusually low.</t>
+        </is>
+      </c>
+      <c r="D19" s="38" t="inlineStr">
+        <is>
+          <t>Could be per-bag, making the line 6x this cost.</t>
+        </is>
+      </c>
+      <c r="E19" s="38" t="inlineStr">
+        <is>
+          <t>Verify pack vs unit pricing before ordering.</t>
         </is>
       </c>
     </row>
@@ -2591,529 +3741,530 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="58" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="58" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="74" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Other Categories — products identified, recipes not yet provided</t>
+          <t>Bar Prep Recipes in Margin Edge (TownHall - Columbus)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>These are NOT part of the smoothie powder prep. They need their recipes before order quantities can be calculated.</t>
+          <t>Pulled 2026-09-29. These are the 23 'TH - Bar Prep' recipes. Mapping order-guide products to these will let the cocktail lines calculate instead of ordering to par.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="34" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="B4" s="34" t="inlineStr">
-        <is>
-          <t>Product</t>
-        </is>
-      </c>
-      <c r="C4" s="34" t="inlineStr">
-        <is>
-          <t>Pack Size</t>
-        </is>
-      </c>
-      <c r="D4" s="34" t="inlineStr">
-        <is>
-          <t>Price</t>
-        </is>
-      </c>
-      <c r="E4" s="34" t="inlineStr">
-        <is>
-          <t>Used In / Note</t>
+      <c r="A4" s="35" t="inlineStr">
+        <is>
+          <t>Recipe ID</t>
+        </is>
+      </c>
+      <c r="B4" s="35" t="inlineStr">
+        <is>
+          <t>Recipe</t>
+        </is>
+      </c>
+      <c r="C4" s="35" t="inlineStr">
+        <is>
+          <t>Cost</t>
+        </is>
+      </c>
+      <c r="D4" s="35" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="E4" s="35" t="inlineStr">
+        <is>
+          <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>Cafe</t>
-        </is>
+      <c r="A5" s="39" t="n">
+        <v>333495432</v>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Anthony's Organic Cacao Cocoa Nibs, Criollo, 2 lb</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>907 g</t>
-        </is>
-      </c>
-      <c r="D5" s="15" t="n">
-        <v>34.99</v>
-      </c>
-      <c r="E5" s="38" t="inlineStr">
-        <is>
-          <t>Acai bowl. Cheaper per gram than Viva ($0.0386 vs $0.0427).</t>
-        </is>
-      </c>
+          <t>Against Doctor's Orders #1 - Batch</t>
+        </is>
+      </c>
+      <c r="C5" s="15" t="n">
+        <v>82.48</v>
+      </c>
+      <c r="D5" s="40" t="inlineStr">
+        <is>
+          <t>128 fl oz</t>
+        </is>
+      </c>
+      <c r="E5" s="41" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>Cafe</t>
-        </is>
+      <c r="A6" s="39" t="n">
+        <v>333490741</v>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Viva Naturals Organic Cacao Nibs, unsweetened, 1 lb</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>454 g</t>
-        </is>
-      </c>
-      <c r="D6" s="15" t="n">
-        <v>19.39</v>
-      </c>
-      <c r="E6" s="38" t="inlineStr">
-        <is>
-          <t>Acai bowl. Second nib SKU — confirm both are needed.</t>
+          <t>Apple Cinnamon Infused Bacardi</t>
+        </is>
+      </c>
+      <c r="C6" s="15" t="n">
+        <v>28.8</v>
+      </c>
+      <c r="D6" s="40" t="inlineStr">
+        <is>
+          <t>24.5 fl oz</t>
+        </is>
+      </c>
+      <c r="E6" s="41" t="inlineStr">
+        <is>
+          <t>Spirit infusion — liquor vendor</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>Smoothie Liquid Mix</t>
-        </is>
+      <c r="A7" s="39" t="n">
+        <v>333478898</v>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Nature's Greatest Organic Coconut Cream, no guar gum</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>12 x 13.5 fl oz</t>
-        </is>
-      </c>
-      <c r="D7" s="15" t="n">
-        <v>45.44</v>
-      </c>
-      <c r="E7" s="38" t="inlineStr">
-        <is>
-          <t>CONFIRMED in Margin Edge: Being Brigid Liquid Mix.</t>
-        </is>
-      </c>
+          <t>At Dawn They Sleep - Batch</t>
+        </is>
+      </c>
+      <c r="C7" s="15" t="n">
+        <v>25.48</v>
+      </c>
+      <c r="D7" s="40" t="inlineStr">
+        <is>
+          <t>34 fl oz</t>
+        </is>
+      </c>
+      <c r="E7" s="41" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>Smoothie Liquid Mix</t>
-        </is>
+      <c r="A8" s="39" t="n">
+        <v>328403264</v>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Mooala Organic Simple Almond Milk, unsweetened</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>6 x 32 oz</t>
-        </is>
-      </c>
-      <c r="D8" s="15" t="n">
-        <v>36.99</v>
-      </c>
-      <c r="E8" s="38" t="inlineStr">
-        <is>
-          <t>Liquid Mix component (per Margin Edge structure).</t>
-        </is>
-      </c>
+          <t>Bloody Mary Spice Blend</t>
+        </is>
+      </c>
+      <c r="C8" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="40" t="inlineStr">
+        <is>
+          <t>8.3 tbsp</t>
+        </is>
+      </c>
+      <c r="E8" s="41" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>Smoothie Liquid Mix</t>
-        </is>
+      <c r="A9" s="39" t="n">
+        <v>333469888</v>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>JOI Instant Oat Milk Creamer Pouch</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>32 servings</t>
-        </is>
-      </c>
-      <c r="D9" s="15" t="n">
-        <v>30.56</v>
-      </c>
-      <c r="E9" s="38" t="inlineStr">
-        <is>
-          <t>Liquid Mix component.</t>
+          <t>Brewed Chai Tea</t>
+        </is>
+      </c>
+      <c r="C9" s="15" t="n">
+        <v>12.91</v>
+      </c>
+      <c r="D9" s="40" t="inlineStr">
+        <is>
+          <t>32 fl oz</t>
+        </is>
+      </c>
+      <c r="E9" s="41" t="inlineStr">
+        <is>
+          <t>USES: Loose Leaf Chai 4 fl oz, Water 32 fl oz, Honey 2 fl oz</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Smoothie Liquid Mix</t>
-        </is>
+      <c r="A10" s="39" t="n">
+        <v>333468674</v>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Nature's Way Organic MCT Oil</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>30 fl oz</t>
-        </is>
-      </c>
-      <c r="D10" s="15" t="n">
-        <v>20.17</v>
-      </c>
-      <c r="E10" s="38" t="inlineStr">
-        <is>
-          <t>Liquid Mix component.</t>
-        </is>
-      </c>
+          <t>Channel Orange - Batched</t>
+        </is>
+      </c>
+      <c r="C10" s="15" t="n">
+        <v>30.78</v>
+      </c>
+      <c r="D10" s="40" t="inlineStr">
+        <is>
+          <t>32 fl oz</t>
+        </is>
+      </c>
+      <c r="E10" s="41" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>Smoothie Liquid Mix</t>
-        </is>
+      <c r="A11" s="39" t="n">
+        <v>333464610</v>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Equip Foods Prime Protein, Vanilla (grass-fed beef)</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>30 servings</t>
-        </is>
-      </c>
-      <c r="D11" s="15" t="n">
-        <v>64.63</v>
-      </c>
-      <c r="E11" s="38" t="inlineStr">
-        <is>
-          <t>Liquid Mix component.</t>
-        </is>
-      </c>
+          <t>Crash Course - Batched</t>
+        </is>
+      </c>
+      <c r="C11" s="15" t="n">
+        <v>26.19</v>
+      </c>
+      <c r="D11" s="40" t="inlineStr">
+        <is>
+          <t>32 fl oz</t>
+        </is>
+      </c>
+      <c r="E11" s="41" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>Cocktail / Bar</t>
-        </is>
+      <c r="A12" s="39" t="n">
+        <v>333504278</v>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Blue Green Organics Raw Blue Agave Syrup</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>176 oz</t>
-        </is>
-      </c>
-      <c r="D12" s="15" t="n">
-        <v>45.59</v>
-      </c>
-      <c r="E12" s="38" t="inlineStr">
-        <is>
-          <t>Awaiting cocktail recipes.</t>
+          <t>Dragonwell Infused OYO Vodka</t>
+        </is>
+      </c>
+      <c r="C12" s="15" t="n">
+        <v>16.45</v>
+      </c>
+      <c r="D12" s="40" t="inlineStr">
+        <is>
+          <t>24 fl oz</t>
+        </is>
+      </c>
+      <c r="E12" s="41" t="inlineStr">
+        <is>
+          <t>Spirit infusion — liquor vendor</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>Cocktail / Bar</t>
-        </is>
+      <c r="A13" s="39" t="n">
+        <v>333500998</v>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Simply Organic Vanilla Bean Paste</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>4 oz jar</t>
-        </is>
-      </c>
-      <c r="D13" s="15" t="n">
-        <v>17.89</v>
-      </c>
-      <c r="E13" s="38" t="inlineStr">
-        <is>
-          <t>Qty 10 ordered — likely a batched syrup component.</t>
-        </is>
-      </c>
+          <t>Espresso Martini Mix</t>
+        </is>
+      </c>
+      <c r="C13" s="15" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="D13" s="40" t="inlineStr">
+        <is>
+          <t>25.4 fl oz</t>
+        </is>
+      </c>
+      <c r="E13" s="41" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>Cocktail / Bar</t>
-        </is>
+      <c r="A14" s="39" t="n">
+        <v>333492968</v>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Bhakti Chai Tea Concentrate, Unsweetened</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>2-pack, 16 srv</t>
-        </is>
-      </c>
-      <c r="D14" s="15" t="n">
-        <v>19.99</v>
-      </c>
-      <c r="E14" s="38" t="inlineStr">
-        <is>
-          <t>Two chai formats in rotation — confirm both are needed.</t>
+          <t>Fall Coconut Cream</t>
+        </is>
+      </c>
+      <c r="C14" s="15" t="n">
+        <v>18.14</v>
+      </c>
+      <c r="D14" s="40" t="inlineStr">
+        <is>
+          <t>72 fl oz</t>
+        </is>
+      </c>
+      <c r="E14" s="41" t="inlineStr">
+        <is>
+          <t>USES: Coconut Cream 15 fl oz, Coconut Milk 13.5 fl oz, pineapple, allspice, cinnamon, nutmeg, pom molasses</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>Cocktail / Bar</t>
-        </is>
+      <c r="A15" s="39" t="n">
+        <v>333473987</v>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Davidson's Tea Bulk, Classic Chai</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>16 oz</t>
-        </is>
-      </c>
-      <c r="D15" s="15" t="n">
-        <v>19.12</v>
-      </c>
-      <c r="E15" s="38" t="inlineStr">
-        <is>
-          <t>Loose leaf, not concentrate.</t>
+          <t>Grapefruit Infused Patron</t>
+        </is>
+      </c>
+      <c r="C15" s="15" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="D15" s="40" t="inlineStr">
+        <is>
+          <t>1 bottle</t>
+        </is>
+      </c>
+      <c r="E15" s="41" t="inlineStr">
+        <is>
+          <t>Spirit infusion — cost looks wrong ($0.06)</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>Cocktail / Bar</t>
-        </is>
+      <c r="A16" s="39" t="n">
+        <v>333504038</v>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Organic Hibiscus Flowers, cut &amp; sifted</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>2 lb</t>
-        </is>
-      </c>
-      <c r="D16" s="15" t="n">
-        <v>27.51</v>
-      </c>
-      <c r="E16" s="38" t="inlineStr">
-        <is>
-          <t>Awaiting recipe.</t>
-        </is>
-      </c>
+          <t>Green Goddess - Batch</t>
+        </is>
+      </c>
+      <c r="C16" s="15" t="n">
+        <v>18.55</v>
+      </c>
+      <c r="D16" s="40" t="inlineStr">
+        <is>
+          <t>33 fl oz</t>
+        </is>
+      </c>
+      <c r="E16" s="41" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>Cocktail / Bar</t>
-        </is>
+      <c r="A17" s="39" t="n">
+        <v>525737107</v>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Frontier Co-op Organic Whole Star Anise</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>1 lb</t>
-        </is>
-      </c>
-      <c r="D17" s="15" t="n">
-        <v>33.52</v>
-      </c>
-      <c r="E17" s="38" t="inlineStr">
-        <is>
-          <t>Awaiting recipe.</t>
-        </is>
-      </c>
+          <t>Heaven or LV BIZ - TH</t>
+        </is>
+      </c>
+      <c r="C17" s="15" t="n">
+        <v>7.28</v>
+      </c>
+      <c r="D17" s="40" t="inlineStr">
+        <is>
+          <t>4.5 fl oz</t>
+        </is>
+      </c>
+      <c r="E17" s="41" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>Cocktail / Bar</t>
-        </is>
+      <c r="A18" s="39" t="n">
+        <v>333481247</v>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Frontier Organic Pumpkin Pie Spice</t>
-        </is>
-      </c>
-      <c r="C18" s="4" t="inlineStr">
-        <is>
-          <t>16 oz</t>
-        </is>
-      </c>
-      <c r="D18" s="15" t="n">
-        <v>13.12</v>
-      </c>
-      <c r="E18" s="38" t="inlineStr">
-        <is>
-          <t>NOT the Longevity cinnamon — that's a blend.</t>
-        </is>
-      </c>
+          <t>Jammy Pom Juice</t>
+        </is>
+      </c>
+      <c r="C18" s="15" t="n">
+        <v>8.199999999999999</v>
+      </c>
+      <c r="D18" s="40" t="inlineStr">
+        <is>
+          <t>35 fl oz</t>
+        </is>
+      </c>
+      <c r="E18" s="41" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>Unassigned</t>
-        </is>
+      <c r="A19" s="39" t="n">
+        <v>333486093</v>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Yupik Organic Raw Pecans</t>
-        </is>
-      </c>
-      <c r="C19" s="4" t="inlineStr">
-        <is>
-          <t>2.2 lb</t>
-        </is>
-      </c>
-      <c r="D19" s="15" t="n">
-        <v>39.93</v>
-      </c>
-      <c r="E19" s="38" t="inlineStr">
-        <is>
-          <t>No recipe yet.</t>
-        </is>
-      </c>
+          <t>Lemony Lemon Curd Juice</t>
+        </is>
+      </c>
+      <c r="C19" s="15" t="n">
+        <v>2.42</v>
+      </c>
+      <c r="D19" s="40" t="inlineStr">
+        <is>
+          <t>25 fl oz</t>
+        </is>
+      </c>
+      <c r="E19" s="41" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>Unassigned</t>
-        </is>
+      <c r="A20" s="39" t="n">
+        <v>333470550</v>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>MADHAVA Organic Coconut Sugar</t>
-        </is>
-      </c>
-      <c r="C20" s="4" t="inlineStr">
-        <is>
-          <t>6 x 1 lb</t>
-        </is>
-      </c>
-      <c r="D20" s="15" t="n">
-        <v>14.26</v>
-      </c>
-      <c r="E20" s="38" t="inlineStr">
-        <is>
-          <t>Verify whether price is per-pack or per-unit.</t>
+          <t>Pear Chai Tea</t>
+        </is>
+      </c>
+      <c r="C20" s="15" t="n">
+        <v>8.880000000000001</v>
+      </c>
+      <c r="D20" s="40" t="inlineStr">
+        <is>
+          <t>34 fl oz</t>
+        </is>
+      </c>
+      <c r="E20" s="41" t="inlineStr">
+        <is>
+          <t>USES: Pear Simple Syrup, Brewed Chai Tea, Lemon Juice</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>Unassigned</t>
-        </is>
+      <c r="A21" s="39" t="n">
+        <v>333504478</v>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Annie's Organic Honey Graham Crackers</t>
-        </is>
-      </c>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>14.4 oz</t>
-        </is>
-      </c>
-      <c r="D21" s="15" t="n">
-        <v>5</v>
-      </c>
-      <c r="E21" s="38" t="inlineStr">
-        <is>
-          <t>No recipe yet.</t>
-        </is>
-      </c>
+          <t>Spicy Cucumber Juice</t>
+        </is>
+      </c>
+      <c r="C21" s="15" t="n">
+        <v>7.18</v>
+      </c>
+      <c r="D21" s="40" t="inlineStr">
+        <is>
+          <t>33.25 fl oz</t>
+        </is>
+      </c>
+      <c r="E21" s="41" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="4" t="inlineStr">
-        <is>
-          <t>Unassigned</t>
-        </is>
+      <c r="A22" s="39" t="n">
+        <v>333485862</v>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Lakanto Peanut Butter Powder, monk-fruit sweetened</t>
-        </is>
-      </c>
-      <c r="C22" s="4" t="inlineStr">
-        <is>
-          <t>8.5 oz</t>
-        </is>
-      </c>
-      <c r="D22" s="15" t="n">
-        <v>13.36</v>
-      </c>
-      <c r="E22" s="38" t="inlineStr">
-        <is>
-          <t>NOT the smoothie PB powder. Keep separate from prep stock.</t>
+          <t>Strawberry Infused Bombay Bramble</t>
+        </is>
+      </c>
+      <c r="C22" s="15" t="n">
+        <v>22.33</v>
+      </c>
+      <c r="D22" s="40" t="inlineStr">
+        <is>
+          <t>24.5 fl oz</t>
+        </is>
+      </c>
+      <c r="E22" s="41" t="inlineStr">
+        <is>
+          <t>Spirit infusion — liquor vendor</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="4" t="inlineStr">
-        <is>
-          <t>Unassigned</t>
-        </is>
+      <c r="A23" s="39" t="n">
+        <v>333486498</v>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Orgain Hydrolyzed Collagen Peptides, Unflavored</t>
-        </is>
-      </c>
-      <c r="C23" s="4" t="inlineStr">
-        <is>
-          <t>454 g</t>
-        </is>
-      </c>
-      <c r="D23" s="15" t="n">
-        <v>21.12</v>
-      </c>
-      <c r="E23" s="38" t="inlineStr">
-        <is>
-          <t>Bought 9/21 but not in any powder prep recipe.</t>
+          <t>Strawberry Kush - Batch</t>
+        </is>
+      </c>
+      <c r="C23" s="15" t="n">
+        <v>33.51</v>
+      </c>
+      <c r="D23" s="40" t="inlineStr">
+        <is>
+          <t>40 fl oz</t>
+        </is>
+      </c>
+      <c r="E23" s="41" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="39" t="n">
+        <v>333498796</v>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>Sweetheart Infused Vodka</t>
+        </is>
+      </c>
+      <c r="C24" s="15" t="n">
+        <v>19.72</v>
+      </c>
+      <c r="D24" s="40" t="inlineStr">
+        <is>
+          <t>27 fl oz</t>
+        </is>
+      </c>
+      <c r="E24" s="41" t="inlineStr">
+        <is>
+          <t>Spirit infusion — liquor vendor</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="39" t="n">
+        <v>333504145</v>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>Syrup, Arugula</t>
+        </is>
+      </c>
+      <c r="C25" s="15" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="D25" s="40" t="inlineStr">
+        <is>
+          <t>12 fl oz</t>
+        </is>
+      </c>
+      <c r="E25" s="41" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="39" t="n">
+        <v>333468799</v>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>Syrup, Pear Simple</t>
+        </is>
+      </c>
+      <c r="C26" s="15" t="n">
+        <v>8.470000000000001</v>
+      </c>
+      <c r="D26" s="40" t="inlineStr">
+        <is>
+          <t>32 fl oz</t>
+        </is>
+      </c>
+      <c r="E26" s="41" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="39" t="n">
+        <v>333460643</v>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>Syrup, Queen of Earl</t>
+        </is>
+      </c>
+      <c r="C27" s="15" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="D27" s="40" t="inlineStr">
+        <is>
+          <t>16 fl oz</t>
+        </is>
+      </c>
+      <c r="E27" s="41" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="9" t="inlineStr">
+        <is>
+          <t>Only 3 of the 23 had their ingredient lists pulled (noted above). Hibiscus syrups sit under 'TH - Prep', not 'TH - Bar Prep'.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add all 23 bar prep recipes and their purchased goods
Pull the full ingredient list for every TH - Bar Prep recipe in Margin
Edge and add a Bar Prep Reference tab showing each recipe with its
ingredients classified as spirit, produce, dry spice, purchased good,
sub-recipe or water.

Add the 21 purchased goods those recipes consume to the order guide as
a new section: juices, honey, demerara, orgeat, preserves, teas,
bitters, coconut milk and cold brew. They need vendor and pack data
before they can calculate, so they carry no price yet.

The pull also surfaced more data errors: a bottle of Patron Silver
costed at $0.06, the Columbus water charge appearing in two more bar
recipes, and five purchased goods costed at zero.

Order guide is now 61 product lines across 8 sections.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01W5WUQdsyFygtfJrtmcjz3J
</commit_message>
<xml_diff>
--- a/order-guide/TownHall-Order-Guide.xlsx
+++ b/order-guide/TownHall-Order-Guide.xlsx
@@ -23,7 +23,7 @@
     <numFmt numFmtId="164" formatCode="$#,##0.00;($#,##0.00);-"/>
     <numFmt numFmtId="165" formatCode="$0.0000"/>
   </numFmts>
-  <fonts count="18">
+  <fonts count="20">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -123,8 +123,19 @@
       <name val="Arial"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00C00000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00C00000"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -149,6 +160,31 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFFF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
   </fills>
@@ -178,7 +214,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -242,13 +278,34 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1073,7 +1130,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M63"/>
+  <dimension ref="A1:M85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2923,7 +2980,7 @@
     <row r="45">
       <c r="A45" s="12" t="inlineStr">
         <is>
-          <t>CAFE</t>
+          <t>COCKTAIL / BAR — PURCHASED GOODS from Margin Edge bar prep recipes (need vendor + pack to become orderable)</t>
         </is>
       </c>
       <c r="B45" s="13" t="n"/>
@@ -2942,237 +2999,227 @@
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>Cacao Nibs</t>
+          <t>Juice, Lemon</t>
         </is>
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>Anthony's Organic Cacao Cocoa Nibs, Criollo, 2 lb</t>
+          <t>Juice, Lemon (ME product 170601314)</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Margin Edge</t>
         </is>
       </c>
       <c r="D46" s="14" t="inlineStr">
         <is>
-          <t>907 g</t>
-        </is>
-      </c>
-      <c r="E46" s="15" t="n">
-        <v>34.99</v>
-      </c>
-      <c r="F46" s="16">
-        <f>IFERROR(E46/907,"")</f>
-        <v/>
-      </c>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E46" s="24" t="n"/>
+      <c r="F46" s="24" t="n"/>
       <c r="G46" s="24" t="n"/>
       <c r="H46" s="24" t="n"/>
-      <c r="I46" s="19" t="n"/>
-      <c r="J46" s="25" t="inlineStr">
-        <is>
-          <t>par</t>
-        </is>
-      </c>
-      <c r="K46" s="19" t="n"/>
-      <c r="L46" s="20">
-        <f>IFERROR(N(K46)*E46,0)</f>
-        <v/>
-      </c>
+      <c r="I46" s="24" t="n"/>
+      <c r="J46" s="24" t="n"/>
+      <c r="K46" s="24" t="n"/>
+      <c r="L46" s="24" t="n"/>
       <c r="M46" s="21" t="inlineStr">
         <is>
-          <t>Acai bowl. Cheaper per gram than Viva ($0.0386 vs $0.0427).</t>
+          <t>4 bar prep recipes — $2.42 per 20 fl oz in use</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>Cacao Nibs (alt)</t>
+          <t>Juice, Lime</t>
         </is>
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>Viva Naturals Organic Cacao Nibs, unsweetened, 1 lb</t>
+          <t>Juice, Lime (ME product 170601652)</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Margin Edge</t>
         </is>
       </c>
       <c r="D47" s="14" t="inlineStr">
         <is>
-          <t>454 g</t>
-        </is>
-      </c>
-      <c r="E47" s="15" t="n">
-        <v>19.39</v>
-      </c>
-      <c r="F47" s="16">
-        <f>IFERROR(E47/454,"")</f>
-        <v/>
-      </c>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E47" s="24" t="n"/>
+      <c r="F47" s="24" t="n"/>
       <c r="G47" s="24" t="n"/>
       <c r="H47" s="24" t="n"/>
-      <c r="I47" s="19" t="n"/>
-      <c r="J47" s="25" t="inlineStr">
-        <is>
-          <t>par</t>
-        </is>
-      </c>
-      <c r="K47" s="19" t="n"/>
-      <c r="L47" s="20">
-        <f>IFERROR(N(K47)*E47,0)</f>
-        <v/>
-      </c>
+      <c r="I47" s="24" t="n"/>
+      <c r="J47" s="24" t="n"/>
+      <c r="K47" s="24" t="n"/>
+      <c r="L47" s="24" t="n"/>
       <c r="M47" s="21" t="inlineStr">
         <is>
-          <t>Acai bowl. Second nib SKU — confirm both are needed.</t>
+          <t>Heaven or LV</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="12" t="inlineStr">
-        <is>
-          <t>UNASSIGNED — bought, but not tied to a recipe. Do not order until confirmed.</t>
-        </is>
-      </c>
-      <c r="B48" s="13" t="n"/>
-      <c r="C48" s="13" t="n"/>
-      <c r="D48" s="13" t="n"/>
-      <c r="E48" s="13" t="n"/>
-      <c r="F48" s="13" t="n"/>
-      <c r="G48" s="13" t="n"/>
-      <c r="H48" s="13" t="n"/>
-      <c r="I48" s="13" t="n"/>
-      <c r="J48" s="13" t="n"/>
-      <c r="K48" s="13" t="n"/>
-      <c r="L48" s="13" t="n"/>
-      <c r="M48" s="13" t="n"/>
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>Juice, Pineapple</t>
+        </is>
+      </c>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>Juice, Pineapple (ME product 171725183)</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>Margin Edge</t>
+        </is>
+      </c>
+      <c r="D48" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E48" s="24" t="n"/>
+      <c r="F48" s="24" t="n"/>
+      <c r="G48" s="24" t="n"/>
+      <c r="H48" s="24" t="n"/>
+      <c r="I48" s="24" t="n"/>
+      <c r="J48" s="24" t="n"/>
+      <c r="K48" s="24" t="n"/>
+      <c r="L48" s="24" t="n"/>
+      <c r="M48" s="21" t="inlineStr">
+        <is>
+          <t>Heaven or LV; Fall Coconut Cream uses a sub-recipe version</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>Peanut Butter Powder (sweetened)</t>
+          <t>Juice, Grapefruit</t>
         </is>
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>Lakanto Peanut Butter Powder, monk-fruit sweetened</t>
+          <t>Juice, Grapefruit (ME product 219558657)</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Margin Edge</t>
         </is>
       </c>
       <c r="D49" s="14" t="inlineStr">
         <is>
-          <t>8.5 oz</t>
-        </is>
-      </c>
-      <c r="E49" s="15" t="n">
-        <v>13.36</v>
-      </c>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E49" s="24" t="n"/>
       <c r="F49" s="24" t="n"/>
       <c r="G49" s="24" t="n"/>
       <c r="H49" s="24" t="n"/>
-      <c r="I49" s="19" t="n"/>
-      <c r="J49" s="25" t="inlineStr">
-        <is>
-          <t>par</t>
-        </is>
-      </c>
-      <c r="K49" s="19" t="n"/>
-      <c r="L49" s="20">
-        <f>IFERROR(N(K49)*E49,0)</f>
-        <v/>
-      </c>
-      <c r="M49" s="22" t="inlineStr">
-        <is>
-          <t>NOT the smoothie PB powder. Store apart from prep stock to avoid a mix-up.</t>
+      <c r="I49" s="24" t="n"/>
+      <c r="J49" s="24" t="n"/>
+      <c r="K49" s="24" t="n"/>
+      <c r="L49" s="24" t="n"/>
+      <c r="M49" s="21" t="inlineStr">
+        <is>
+          <t>Against Doctor's Orders — $9.75 per 31 fl oz in use</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>Collagen Peptides, Unflavored</t>
+          <t>Juice, Pomegranate</t>
         </is>
       </c>
       <c r="B50" s="4" t="inlineStr">
         <is>
-          <t>Orgain Hydrolyzed Collagen Peptides, Unflavored, 1 lb</t>
+          <t>Juice, Pomegranate (ME product 185463517)</t>
         </is>
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Margin Edge</t>
         </is>
       </c>
       <c r="D50" s="14" t="inlineStr">
         <is>
-          <t>454 g</t>
-        </is>
-      </c>
-      <c r="E50" s="15" t="n">
-        <v>21.12</v>
-      </c>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E50" s="24" t="n"/>
       <c r="F50" s="24" t="n"/>
       <c r="G50" s="24" t="n"/>
       <c r="H50" s="24" t="n"/>
-      <c r="I50" s="19" t="n"/>
-      <c r="J50" s="25" t="inlineStr">
-        <is>
-          <t>par</t>
-        </is>
-      </c>
-      <c r="K50" s="19" t="n"/>
-      <c r="L50" s="20">
-        <f>IFERROR(N(K50)*E50,0)</f>
-        <v/>
-      </c>
-      <c r="M50" s="22" t="inlineStr">
-        <is>
-          <t>Bought 9/21/2026 but appears in no powder prep recipe. Identify the use.</t>
+      <c r="I50" s="24" t="n"/>
+      <c r="J50" s="24" t="n"/>
+      <c r="K50" s="24" t="n"/>
+      <c r="L50" s="24" t="n"/>
+      <c r="M50" s="21" t="inlineStr">
+        <is>
+          <t>Jammy Pom Juice — $3.12 per 20 fl oz</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="12" t="inlineStr">
-        <is>
-          <t>IN-HOUSE — NOT AN ORDER LINE</t>
-        </is>
-      </c>
-      <c r="B51" s="13" t="n"/>
-      <c r="C51" s="13" t="n"/>
-      <c r="D51" s="13" t="n"/>
-      <c r="E51" s="13" t="n"/>
-      <c r="F51" s="13" t="n"/>
-      <c r="G51" s="13" t="n"/>
-      <c r="H51" s="13" t="n"/>
-      <c r="I51" s="13" t="n"/>
-      <c r="J51" s="13" t="n"/>
-      <c r="K51" s="13" t="n"/>
-      <c r="L51" s="13" t="n"/>
-      <c r="M51" s="13" t="n"/>
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Honey</t>
+        </is>
+      </c>
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>Honey (ME product 173336779)</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="inlineStr">
+        <is>
+          <t>Margin Edge</t>
+        </is>
+      </c>
+      <c r="D51" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E51" s="24" t="n"/>
+      <c r="F51" s="24" t="n"/>
+      <c r="G51" s="24" t="n"/>
+      <c r="H51" s="24" t="n"/>
+      <c r="I51" s="24" t="n"/>
+      <c r="J51" s="24" t="n"/>
+      <c r="K51" s="24" t="n"/>
+      <c r="L51" s="24" t="n"/>
+      <c r="M51" s="21" t="inlineStr">
+        <is>
+          <t>Brewed Chai Tea, Heaven or LV</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
         <is>
-          <t>Cinnamon, Ground</t>
+          <t>Sugar, Demerara</t>
         </is>
       </c>
       <c r="B52" s="4" t="inlineStr">
         <is>
-          <t>Carried in kitchen stock</t>
+          <t>Sugar, Demerara (ME product 321915601)</t>
         </is>
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t>In-house</t>
+          <t>Margin Edge</t>
         </is>
       </c>
       <c r="D52" s="14" t="inlineStr">
@@ -3182,10 +3229,7 @@
       </c>
       <c r="E52" s="24" t="n"/>
       <c r="F52" s="24" t="n"/>
-      <c r="G52" s="17">
-        <f>'Recipe Usage'!F24</f>
-        <v/>
-      </c>
+      <c r="G52" s="24" t="n"/>
       <c r="H52" s="24" t="n"/>
       <c r="I52" s="24" t="n"/>
       <c r="J52" s="24" t="n"/>
@@ -3193,83 +3237,850 @@
       <c r="L52" s="24" t="n"/>
       <c r="M52" s="21" t="inlineStr">
         <is>
+          <t>Syrup Queen of Earl — $6.30 per 454 g</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>Syrup, Orgeat</t>
+        </is>
+      </c>
+      <c r="B53" s="4" t="inlineStr">
+        <is>
+          <t>Syrup, Orgeat (ME product 302352282)</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="inlineStr">
+        <is>
+          <t>Margin Edge</t>
+        </is>
+      </c>
+      <c r="D53" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E53" s="24" t="n"/>
+      <c r="F53" s="24" t="n"/>
+      <c r="G53" s="24" t="n"/>
+      <c r="H53" s="24" t="n"/>
+      <c r="I53" s="24" t="n"/>
+      <c r="J53" s="24" t="n"/>
+      <c r="K53" s="24" t="n"/>
+      <c r="L53" s="24" t="n"/>
+      <c r="M53" s="21" t="inlineStr">
+        <is>
+          <t>Strawberry Kush — $7.80 per 11 fl oz</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>Molasses, Pomegranate</t>
+        </is>
+      </c>
+      <c r="B54" s="4" t="inlineStr">
+        <is>
+          <t>Molasses, Pomegranate (ME product 174116373)</t>
+        </is>
+      </c>
+      <c r="C54" s="4" t="inlineStr">
+        <is>
+          <t>Margin Edge</t>
+        </is>
+      </c>
+      <c r="D54" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E54" s="24" t="n"/>
+      <c r="F54" s="24" t="n"/>
+      <c r="G54" s="24" t="n"/>
+      <c r="H54" s="24" t="n"/>
+      <c r="I54" s="24" t="n"/>
+      <c r="J54" s="24" t="n"/>
+      <c r="K54" s="24" t="n"/>
+      <c r="L54" s="24" t="n"/>
+      <c r="M54" s="21" t="inlineStr">
+        <is>
+          <t>Fall Coconut Cream</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Preserves, Lingonberry</t>
+        </is>
+      </c>
+      <c r="B55" s="4" t="inlineStr">
+        <is>
+          <t>Preserves, Lingonberry (ME product 311107139)</t>
+        </is>
+      </c>
+      <c r="C55" s="4" t="inlineStr">
+        <is>
+          <t>Margin Edge</t>
+        </is>
+      </c>
+      <c r="D55" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E55" s="24" t="n"/>
+      <c r="F55" s="24" t="n"/>
+      <c r="G55" s="24" t="n"/>
+      <c r="H55" s="24" t="n"/>
+      <c r="I55" s="24" t="n"/>
+      <c r="J55" s="24" t="n"/>
+      <c r="K55" s="24" t="n"/>
+      <c r="L55" s="24" t="n"/>
+      <c r="M55" s="21" t="inlineStr">
+        <is>
+          <t>Jammy Pom Juice — $3.14 per 5 fl oz</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Preserves, Lemon Curd</t>
+        </is>
+      </c>
+      <c r="B56" s="4" t="inlineStr">
+        <is>
+          <t>Preserves, Lemon Curd (ME product 331999220)</t>
+        </is>
+      </c>
+      <c r="C56" s="4" t="inlineStr">
+        <is>
+          <t>Margin Edge</t>
+        </is>
+      </c>
+      <c r="D56" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E56" s="24" t="n"/>
+      <c r="F56" s="24" t="n"/>
+      <c r="G56" s="24" t="n"/>
+      <c r="H56" s="24" t="n"/>
+      <c r="I56" s="24" t="n"/>
+      <c r="J56" s="24" t="n"/>
+      <c r="K56" s="24" t="n"/>
+      <c r="L56" s="24" t="n"/>
+      <c r="M56" s="22" t="inlineStr">
+        <is>
+          <t>Lemony Lemon Curd Juice — priced $0.00 in ME, needs a real cost</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>Jelly, Hot Pepper</t>
+        </is>
+      </c>
+      <c r="B57" s="4" t="inlineStr">
+        <is>
+          <t>Jelly, Hot Pepper (ME product 302355790)</t>
+        </is>
+      </c>
+      <c r="C57" s="4" t="inlineStr">
+        <is>
+          <t>Margin Edge</t>
+        </is>
+      </c>
+      <c r="D57" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E57" s="24" t="n"/>
+      <c r="F57" s="24" t="n"/>
+      <c r="G57" s="24" t="n"/>
+      <c r="H57" s="24" t="n"/>
+      <c r="I57" s="24" t="n"/>
+      <c r="J57" s="24" t="n"/>
+      <c r="K57" s="24" t="n"/>
+      <c r="L57" s="24" t="n"/>
+      <c r="M57" s="21" t="inlineStr">
+        <is>
+          <t>Jammy Pom Juice — $1.94 per 5 fl oz</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>Milk, Coconut Canned</t>
+        </is>
+      </c>
+      <c r="B58" s="4" t="inlineStr">
+        <is>
+          <t>Milk, Coconut Canned (ME product 171721565)</t>
+        </is>
+      </c>
+      <c r="C58" s="4" t="inlineStr">
+        <is>
+          <t>Margin Edge</t>
+        </is>
+      </c>
+      <c r="D58" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E58" s="24" t="n"/>
+      <c r="F58" s="24" t="n"/>
+      <c r="G58" s="24" t="n"/>
+      <c r="H58" s="24" t="n"/>
+      <c r="I58" s="24" t="n"/>
+      <c r="J58" s="24" t="n"/>
+      <c r="K58" s="24" t="n"/>
+      <c r="L58" s="24" t="n"/>
+      <c r="M58" s="21" t="inlineStr">
+        <is>
+          <t>Fall Coconut Cream — $1.60 per 13.5 fl oz</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="4" t="inlineStr">
+        <is>
+          <t>Cold Brew Concentrate</t>
+        </is>
+      </c>
+      <c r="B59" s="4" t="inlineStr">
+        <is>
+          <t>Six Shooter Cold Brew, gallon (ME product 177626990)</t>
+        </is>
+      </c>
+      <c r="C59" s="4" t="inlineStr">
+        <is>
+          <t>Margin Edge</t>
+        </is>
+      </c>
+      <c r="D59" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E59" s="24" t="n"/>
+      <c r="F59" s="24" t="n"/>
+      <c r="G59" s="24" t="n"/>
+      <c r="H59" s="24" t="n"/>
+      <c r="I59" s="24" t="n"/>
+      <c r="J59" s="24" t="n"/>
+      <c r="K59" s="24" t="n"/>
+      <c r="L59" s="24" t="n"/>
+      <c r="M59" s="21" t="inlineStr">
+        <is>
+          <t>Espresso Martini Mix — $1.86 per 12.7 fl oz</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="4" t="inlineStr">
+        <is>
+          <t>Tea, Butterfly Pea Flowers</t>
+        </is>
+      </c>
+      <c r="B60" s="4" t="inlineStr">
+        <is>
+          <t>Tea, Butterfly Pea Flowers (ME product 470340233)</t>
+        </is>
+      </c>
+      <c r="C60" s="4" t="inlineStr">
+        <is>
+          <t>Margin Edge</t>
+        </is>
+      </c>
+      <c r="D60" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E60" s="24" t="n"/>
+      <c r="F60" s="24" t="n"/>
+      <c r="G60" s="24" t="n"/>
+      <c r="H60" s="24" t="n"/>
+      <c r="I60" s="24" t="n"/>
+      <c r="J60" s="24" t="n"/>
+      <c r="K60" s="24" t="n"/>
+      <c r="L60" s="24" t="n"/>
+      <c r="M60" s="21" t="inlineStr">
+        <is>
+          <t>Heaven or LV — $5.45 per oz</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="4" t="inlineStr">
+        <is>
+          <t>Tea, Peruvian Spiced Berry</t>
+        </is>
+      </c>
+      <c r="B61" s="4" t="inlineStr">
+        <is>
+          <t>Tea, Peruvian Spiced Berry (ME product 188277776)</t>
+        </is>
+      </c>
+      <c r="C61" s="4" t="inlineStr">
+        <is>
+          <t>Margin Edge</t>
+        </is>
+      </c>
+      <c r="D61" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E61" s="24" t="n"/>
+      <c r="F61" s="24" t="n"/>
+      <c r="G61" s="24" t="n"/>
+      <c r="H61" s="24" t="n"/>
+      <c r="I61" s="24" t="n"/>
+      <c r="J61" s="24" t="n"/>
+      <c r="K61" s="24" t="n"/>
+      <c r="L61" s="24" t="n"/>
+      <c r="M61" s="21" t="inlineStr">
+        <is>
+          <t>Sweetheart Infused Vodka — $2.38 per 2 oz</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="4" t="inlineStr">
+        <is>
+          <t>Tea, Herbal (apple cinnamon)</t>
+        </is>
+      </c>
+      <c r="B62" s="4" t="inlineStr">
+        <is>
+          <t>Tea, Herbal (ME product 176357503)</t>
+        </is>
+      </c>
+      <c r="C62" s="4" t="inlineStr">
+        <is>
+          <t>Margin Edge</t>
+        </is>
+      </c>
+      <c r="D62" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E62" s="24" t="n"/>
+      <c r="F62" s="24" t="n"/>
+      <c r="G62" s="24" t="n"/>
+      <c r="H62" s="24" t="n"/>
+      <c r="I62" s="24" t="n"/>
+      <c r="J62" s="24" t="n"/>
+      <c r="K62" s="24" t="n"/>
+      <c r="L62" s="24" t="n"/>
+      <c r="M62" s="21" t="inlineStr">
+        <is>
+          <t>Apple Cinnamon Infused Bacardi — $0.60 per 3 bags</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="4" t="inlineStr">
+        <is>
+          <t>Bitters, Xocolatl Mole</t>
+        </is>
+      </c>
+      <c r="B63" s="4" t="inlineStr">
+        <is>
+          <t>Bitters, Xocolatl Mole (ME product 299636143)</t>
+        </is>
+      </c>
+      <c r="C63" s="4" t="inlineStr">
+        <is>
+          <t>Margin Edge</t>
+        </is>
+      </c>
+      <c r="D63" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E63" s="24" t="n"/>
+      <c r="F63" s="24" t="n"/>
+      <c r="G63" s="24" t="n"/>
+      <c r="H63" s="24" t="n"/>
+      <c r="I63" s="24" t="n"/>
+      <c r="J63" s="24" t="n"/>
+      <c r="K63" s="24" t="n"/>
+      <c r="L63" s="24" t="n"/>
+      <c r="M63" s="21" t="inlineStr">
+        <is>
+          <t>Crash Course</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="4" t="inlineStr">
+        <is>
+          <t>Bitters, Barkeep Lavender</t>
+        </is>
+      </c>
+      <c r="B64" s="4" t="inlineStr">
+        <is>
+          <t>Bitters, Barkeep Lavender (ME product 303574372)</t>
+        </is>
+      </c>
+      <c r="C64" s="4" t="inlineStr">
+        <is>
+          <t>Margin Edge</t>
+        </is>
+      </c>
+      <c r="D64" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E64" s="24" t="n"/>
+      <c r="F64" s="24" t="n"/>
+      <c r="G64" s="24" t="n"/>
+      <c r="H64" s="24" t="n"/>
+      <c r="I64" s="24" t="n"/>
+      <c r="J64" s="24" t="n"/>
+      <c r="K64" s="24" t="n"/>
+      <c r="L64" s="24" t="n"/>
+      <c r="M64" s="21" t="inlineStr">
+        <is>
+          <t>Crash Course — $1.90 per 0.5 fl oz</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="4" t="inlineStr">
+        <is>
+          <t>Bitters, Orange</t>
+        </is>
+      </c>
+      <c r="B65" s="4" t="inlineStr">
+        <is>
+          <t>Bitters, Orange (ME product 303574872)</t>
+        </is>
+      </c>
+      <c r="C65" s="4" t="inlineStr">
+        <is>
+          <t>Margin Edge</t>
+        </is>
+      </c>
+      <c r="D65" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E65" s="24" t="n"/>
+      <c r="F65" s="24" t="n"/>
+      <c r="G65" s="24" t="n"/>
+      <c r="H65" s="24" t="n"/>
+      <c r="I65" s="24" t="n"/>
+      <c r="J65" s="24" t="n"/>
+      <c r="K65" s="24" t="n"/>
+      <c r="L65" s="24" t="n"/>
+      <c r="M65" s="22" t="inlineStr">
+        <is>
+          <t>Channel Orange — priced $0.00 in ME, needs a real cost</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="4" t="inlineStr">
+        <is>
+          <t>Bitters, Toasted Almond</t>
+        </is>
+      </c>
+      <c r="B66" s="4" t="inlineStr">
+        <is>
+          <t>Bitters, Toasted Almond (ME product 303576251)</t>
+        </is>
+      </c>
+      <c r="C66" s="4" t="inlineStr">
+        <is>
+          <t>Margin Edge</t>
+        </is>
+      </c>
+      <c r="D66" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E66" s="24" t="n"/>
+      <c r="F66" s="24" t="n"/>
+      <c r="G66" s="24" t="n"/>
+      <c r="H66" s="24" t="n"/>
+      <c r="I66" s="24" t="n"/>
+      <c r="J66" s="24" t="n"/>
+      <c r="K66" s="24" t="n"/>
+      <c r="L66" s="24" t="n"/>
+      <c r="M66" s="22" t="inlineStr">
+        <is>
+          <t>Strawberry Kush — priced $0.00 in ME, needs a real cost</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="12" t="inlineStr">
+        <is>
+          <t>CAFE</t>
+        </is>
+      </c>
+      <c r="B67" s="13" t="n"/>
+      <c r="C67" s="13" t="n"/>
+      <c r="D67" s="13" t="n"/>
+      <c r="E67" s="13" t="n"/>
+      <c r="F67" s="13" t="n"/>
+      <c r="G67" s="13" t="n"/>
+      <c r="H67" s="13" t="n"/>
+      <c r="I67" s="13" t="n"/>
+      <c r="J67" s="13" t="n"/>
+      <c r="K67" s="13" t="n"/>
+      <c r="L67" s="13" t="n"/>
+      <c r="M67" s="13" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="4" t="inlineStr">
+        <is>
+          <t>Cacao Nibs</t>
+        </is>
+      </c>
+      <c r="B68" s="4" t="inlineStr">
+        <is>
+          <t>Anthony's Organic Cacao Cocoa Nibs, Criollo, 2 lb</t>
+        </is>
+      </c>
+      <c r="C68" s="4" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D68" s="14" t="inlineStr">
+        <is>
+          <t>907 g</t>
+        </is>
+      </c>
+      <c r="E68" s="15" t="n">
+        <v>34.99</v>
+      </c>
+      <c r="F68" s="16">
+        <f>IFERROR(E68/907,"")</f>
+        <v/>
+      </c>
+      <c r="G68" s="24" t="n"/>
+      <c r="H68" s="24" t="n"/>
+      <c r="I68" s="19" t="n"/>
+      <c r="J68" s="25" t="inlineStr">
+        <is>
+          <t>par</t>
+        </is>
+      </c>
+      <c r="K68" s="19" t="n"/>
+      <c r="L68" s="20">
+        <f>IFERROR(N(K68)*E68,0)</f>
+        <v/>
+      </c>
+      <c r="M68" s="21" t="inlineStr">
+        <is>
+          <t>Acai bowl. Cheaper per gram than Viva ($0.0386 vs $0.0427).</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="4" t="inlineStr">
+        <is>
+          <t>Cacao Nibs (alt)</t>
+        </is>
+      </c>
+      <c r="B69" s="4" t="inlineStr">
+        <is>
+          <t>Viva Naturals Organic Cacao Nibs, unsweetened, 1 lb</t>
+        </is>
+      </c>
+      <c r="C69" s="4" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D69" s="14" t="inlineStr">
+        <is>
+          <t>454 g</t>
+        </is>
+      </c>
+      <c r="E69" s="15" t="n">
+        <v>19.39</v>
+      </c>
+      <c r="F69" s="16">
+        <f>IFERROR(E69/454,"")</f>
+        <v/>
+      </c>
+      <c r="G69" s="24" t="n"/>
+      <c r="H69" s="24" t="n"/>
+      <c r="I69" s="19" t="n"/>
+      <c r="J69" s="25" t="inlineStr">
+        <is>
+          <t>par</t>
+        </is>
+      </c>
+      <c r="K69" s="19" t="n"/>
+      <c r="L69" s="20">
+        <f>IFERROR(N(K69)*E69,0)</f>
+        <v/>
+      </c>
+      <c r="M69" s="21" t="inlineStr">
+        <is>
+          <t>Acai bowl. Second nib SKU — confirm both are needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="12" t="inlineStr">
+        <is>
+          <t>UNASSIGNED — bought, but not tied to a recipe. Do not order until confirmed.</t>
+        </is>
+      </c>
+      <c r="B70" s="13" t="n"/>
+      <c r="C70" s="13" t="n"/>
+      <c r="D70" s="13" t="n"/>
+      <c r="E70" s="13" t="n"/>
+      <c r="F70" s="13" t="n"/>
+      <c r="G70" s="13" t="n"/>
+      <c r="H70" s="13" t="n"/>
+      <c r="I70" s="13" t="n"/>
+      <c r="J70" s="13" t="n"/>
+      <c r="K70" s="13" t="n"/>
+      <c r="L70" s="13" t="n"/>
+      <c r="M70" s="13" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="4" t="inlineStr">
+        <is>
+          <t>Peanut Butter Powder (sweetened)</t>
+        </is>
+      </c>
+      <c r="B71" s="4" t="inlineStr">
+        <is>
+          <t>Lakanto Peanut Butter Powder, monk-fruit sweetened</t>
+        </is>
+      </c>
+      <c r="C71" s="4" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D71" s="14" t="inlineStr">
+        <is>
+          <t>8.5 oz</t>
+        </is>
+      </c>
+      <c r="E71" s="15" t="n">
+        <v>13.36</v>
+      </c>
+      <c r="F71" s="24" t="n"/>
+      <c r="G71" s="24" t="n"/>
+      <c r="H71" s="24" t="n"/>
+      <c r="I71" s="19" t="n"/>
+      <c r="J71" s="25" t="inlineStr">
+        <is>
+          <t>par</t>
+        </is>
+      </c>
+      <c r="K71" s="19" t="n"/>
+      <c r="L71" s="20">
+        <f>IFERROR(N(K71)*E71,0)</f>
+        <v/>
+      </c>
+      <c r="M71" s="22" t="inlineStr">
+        <is>
+          <t>NOT the smoothie PB powder. Store apart from prep stock to avoid a mix-up.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="4" t="inlineStr">
+        <is>
+          <t>Collagen Peptides, Unflavored</t>
+        </is>
+      </c>
+      <c r="B72" s="4" t="inlineStr">
+        <is>
+          <t>Orgain Hydrolyzed Collagen Peptides, Unflavored, 1 lb</t>
+        </is>
+      </c>
+      <c r="C72" s="4" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D72" s="14" t="inlineStr">
+        <is>
+          <t>454 g</t>
+        </is>
+      </c>
+      <c r="E72" s="15" t="n">
+        <v>21.12</v>
+      </c>
+      <c r="F72" s="24" t="n"/>
+      <c r="G72" s="24" t="n"/>
+      <c r="H72" s="24" t="n"/>
+      <c r="I72" s="19" t="n"/>
+      <c r="J72" s="25" t="inlineStr">
+        <is>
+          <t>par</t>
+        </is>
+      </c>
+      <c r="K72" s="19" t="n"/>
+      <c r="L72" s="20">
+        <f>IFERROR(N(K72)*E72,0)</f>
+        <v/>
+      </c>
+      <c r="M72" s="22" t="inlineStr">
+        <is>
+          <t>Bought 9/21/2026 but appears in no powder prep recipe. Identify the use.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="12" t="inlineStr">
+        <is>
+          <t>IN-HOUSE — NOT AN ORDER LINE</t>
+        </is>
+      </c>
+      <c r="B73" s="13" t="n"/>
+      <c r="C73" s="13" t="n"/>
+      <c r="D73" s="13" t="n"/>
+      <c r="E73" s="13" t="n"/>
+      <c r="F73" s="13" t="n"/>
+      <c r="G73" s="13" t="n"/>
+      <c r="H73" s="13" t="n"/>
+      <c r="I73" s="13" t="n"/>
+      <c r="J73" s="13" t="n"/>
+      <c r="K73" s="13" t="n"/>
+      <c r="L73" s="13" t="n"/>
+      <c r="M73" s="13" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="4" t="inlineStr">
+        <is>
+          <t>Cinnamon, Ground</t>
+        </is>
+      </c>
+      <c r="B74" s="4" t="inlineStr">
+        <is>
+          <t>Carried in kitchen stock</t>
+        </is>
+      </c>
+      <c r="C74" s="4" t="inlineStr">
+        <is>
+          <t>In-house</t>
+        </is>
+      </c>
+      <c r="D74" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E74" s="24" t="n"/>
+      <c r="F74" s="24" t="n"/>
+      <c r="G74" s="17">
+        <f>'Recipe Usage'!F24</f>
+        <v/>
+      </c>
+      <c r="H74" s="24" t="n"/>
+      <c r="I74" s="24" t="n"/>
+      <c r="J74" s="24" t="n"/>
+      <c r="K74" s="24" t="n"/>
+      <c r="L74" s="24" t="n"/>
+      <c r="M74" s="21" t="inlineStr">
+        <is>
           <t>Pull from stock. Stays on the prep guide, excluded from ordering.</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="26" t="inlineStr">
+    <row r="75">
+      <c r="A75" s="26" t="inlineStr">
         <is>
           <t>ORDER TOTAL (this location)</t>
         </is>
       </c>
-      <c r="B53" s="27" t="n"/>
-      <c r="C53" s="27" t="n"/>
-      <c r="D53" s="27" t="n"/>
-      <c r="E53" s="27" t="n"/>
-      <c r="F53" s="27" t="n"/>
-      <c r="G53" s="27" t="n"/>
-      <c r="H53" s="27" t="n"/>
-      <c r="I53" s="27" t="n"/>
-      <c r="J53" s="27" t="n"/>
-      <c r="K53" s="27" t="n"/>
-      <c r="L53" s="28">
-        <f>SUM(L6:L52)</f>
-        <v/>
-      </c>
-      <c r="M53" s="27" t="n"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="29" t="inlineStr">
+      <c r="B75" s="27" t="n"/>
+      <c r="C75" s="27" t="n"/>
+      <c r="D75" s="27" t="n"/>
+      <c r="E75" s="27" t="n"/>
+      <c r="F75" s="27" t="n"/>
+      <c r="G75" s="27" t="n"/>
+      <c r="H75" s="27" t="n"/>
+      <c r="I75" s="27" t="n"/>
+      <c r="J75" s="27" t="n"/>
+      <c r="K75" s="27" t="n"/>
+      <c r="L75" s="28">
+        <f>SUM(L6:L74)</f>
+        <v/>
+      </c>
+      <c r="M75" s="27" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="29" t="inlineStr">
         <is>
           <t>LEGEND</t>
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="30" t="inlineStr">
+    <row r="78">
+      <c r="A78" s="30" t="inlineStr">
         <is>
           <t>Yellow cells = you fill in (On Hand, Order Qty)</t>
         </is>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="31" t="inlineStr">
+    <row r="79">
+      <c r="A79" s="31" t="inlineStr">
         <is>
           <t>Blue text = fixed data (pack size, price). Update when prices change.</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="32" t="inlineStr">
+    <row r="80">
+      <c r="A80" s="32" t="inlineStr">
         <is>
           <t>Green text = pulled from the 'Recipe Usage' tab</t>
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" s="30" t="inlineStr">
+    <row r="81">
+      <c r="A81" s="30" t="inlineStr">
         <is>
           <t>Black text = calculated — do not overwrite</t>
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" s="33" t="inlineStr">
+    <row r="82">
+      <c r="A82" s="33" t="inlineStr">
         <is>
           <t>Red text = needs a decision. See the 'Notes &amp; Flags' tab.</t>
         </is>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="34" t="inlineStr">
+    <row r="83">
+      <c r="A83" s="34" t="inlineStr">
         <is>
           <t>"par" in Suggested = no recipe usage mapped yet; order to par by eye until the recipe lands.</t>
         </is>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" s="2" t="inlineStr">
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
         <is>
           <t>EXAMPLE: Chia shows 3 packs/cycle. Enter 1 in On Hand, Suggested reads 2. Enter 2 in Order Qty and Ext. Cost reads $27.94.</t>
         </is>
@@ -3741,530 +4552,2438 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:G109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="38" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="74" customWidth="1" min="5" max="5"/>
+    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Bar Prep Recipes in Margin Edge (TownHall - Columbus)</t>
+          <t>Bar Prep Recipes — TownHall Columbus (Margin Edge, pulled 2026-09-29)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Pulled 2026-09-29. These are the 23 'TH - Bar Prep' recipes. Mapping order-guide products to these will let the cocktail lines calculate instead of ordering to par.</t>
+          <t>All 23 'TH - Bar Prep' recipes with full ingredient lists. Kind: SPIRIT = liquor vendor - PRODUCE = fresh - DRYSPICE = kitchen dry stock - PURCHASED = order-guide candidate - SUBRECIPE = made in house - WATER = should be $0.00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="35" t="inlineStr">
         <is>
-          <t>Recipe ID</t>
+          <t>Recipe / Ingredient</t>
         </is>
       </c>
       <c r="B4" s="35" t="inlineStr">
         <is>
-          <t>Recipe</t>
+          <t>Qty</t>
         </is>
       </c>
       <c r="C4" s="35" t="inlineStr">
         <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="D4" s="35" t="inlineStr">
+        <is>
           <t>Cost</t>
         </is>
       </c>
-      <c r="D4" s="35" t="inlineStr">
+      <c r="E4" s="35" t="inlineStr">
+        <is>
+          <t>Kind</t>
+        </is>
+      </c>
+      <c r="F4" s="35" t="inlineStr">
+        <is>
+          <t>Recipe cost</t>
+        </is>
+      </c>
+      <c r="G4" s="35" t="inlineStr">
         <is>
           <t>Yield</t>
         </is>
       </c>
-      <c r="E4" s="35" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
     </row>
     <row r="5">
-      <c r="A5" s="39" t="n">
-        <v>333495432</v>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Against Doctor's Orders #1 - Batch</t>
         </is>
       </c>
-      <c r="C5" s="15" t="n">
+      <c r="B5" s="13" t="n"/>
+      <c r="C5" s="13" t="n"/>
+      <c r="D5" s="13" t="n"/>
+      <c r="E5" s="13" t="n"/>
+      <c r="F5" s="39" t="n">
         <v>82.48</v>
       </c>
-      <c r="D5" s="40" t="inlineStr">
+      <c r="G5" s="40" t="inlineStr">
         <is>
           <t>128 fl oz</t>
         </is>
       </c>
-      <c r="E5" s="41" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="39" t="n">
-        <v>333490741</v>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Liqueur, Aperol Aperitivo</t>
+        </is>
+      </c>
+      <c r="B6" s="41" t="n">
+        <v>31</v>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>fl oz</t>
+        </is>
+      </c>
+      <c r="D6" s="20" t="n">
+        <v>24.02</v>
+      </c>
+      <c r="E6" s="42" t="inlineStr">
+        <is>
+          <t>SPIRIT</t>
+        </is>
+      </c>
+      <c r="F6" s="24" t="n"/>
+      <c r="G6" s="24" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Gin, Malfy Con Arancia</t>
+        </is>
+      </c>
+      <c r="B7" s="41" t="n">
+        <v>31</v>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>fl oz</t>
+        </is>
+      </c>
+      <c r="D7" s="20" t="n">
+        <v>28.7</v>
+      </c>
+      <c r="E7" s="42" t="inlineStr">
+        <is>
+          <t>SPIRIT</t>
+        </is>
+      </c>
+      <c r="F7" s="24" t="n"/>
+      <c r="G7" s="24" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Juice, Grapefruit</t>
+        </is>
+      </c>
+      <c r="B8" s="41" t="n">
+        <v>31</v>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>fl oz</t>
+        </is>
+      </c>
+      <c r="D8" s="20" t="n">
+        <v>9.75</v>
+      </c>
+      <c r="E8" s="43" t="inlineStr">
+        <is>
+          <t>PURCHASED</t>
+        </is>
+      </c>
+      <c r="F8" s="24" t="n"/>
+      <c r="G8" s="24" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Juice, Lemon</t>
+        </is>
+      </c>
+      <c r="B9" s="41" t="n">
+        <v>15.25</v>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>fl oz</t>
+        </is>
+      </c>
+      <c r="D9" s="20" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="E9" s="43" t="inlineStr">
+        <is>
+          <t>PURCHASED</t>
+        </is>
+      </c>
+      <c r="F9" s="24" t="n"/>
+      <c r="G9" s="24" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Water</t>
+        </is>
+      </c>
+      <c r="B10" s="41" t="n">
+        <v>15.25</v>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>fl oz</t>
+        </is>
+      </c>
+      <c r="D10" s="20" t="n">
+        <v>5.85</v>
+      </c>
+      <c r="E10" s="44" t="inlineStr">
+        <is>
+          <t>WATER</t>
+        </is>
+      </c>
+      <c r="F10" s="24" t="n"/>
+      <c r="G10" s="24" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Kahlua 1L</t>
+        </is>
+      </c>
+      <c r="B11" s="41" t="n">
+        <v>15.25</v>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>fl oz</t>
+        </is>
+      </c>
+      <c r="D11" s="20" t="n">
+        <v>12.31</v>
+      </c>
+      <c r="E11" s="42" t="inlineStr">
+        <is>
+          <t>SPIRIT</t>
+        </is>
+      </c>
+      <c r="F11" s="24" t="n"/>
+      <c r="G11" s="24" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="12" t="inlineStr">
         <is>
           <t>Apple Cinnamon Infused Bacardi</t>
         </is>
       </c>
-      <c r="C6" s="15" t="n">
+      <c r="B12" s="13" t="n"/>
+      <c r="C12" s="13" t="n"/>
+      <c r="D12" s="13" t="n"/>
+      <c r="E12" s="13" t="n"/>
+      <c r="F12" s="39" t="n">
         <v>28.8</v>
       </c>
-      <c r="D6" s="40" t="inlineStr">
+      <c r="G12" s="40" t="inlineStr">
         <is>
           <t>24.5 fl oz</t>
         </is>
       </c>
-      <c r="E6" s="41" t="inlineStr">
-        <is>
-          <t>Spirit infusion — liquor vendor</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="39" t="n">
-        <v>333478898</v>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Bacardi Reserva Ocho</t>
+        </is>
+      </c>
+      <c r="B13" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>bottle</t>
+        </is>
+      </c>
+      <c r="D13" s="20" t="n">
+        <v>28.2</v>
+      </c>
+      <c r="E13" s="42" t="inlineStr">
+        <is>
+          <t>SPIRIT</t>
+        </is>
+      </c>
+      <c r="F13" s="24" t="n"/>
+      <c r="G13" s="24" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Tea, Herbal (apple cinnamon)</t>
+        </is>
+      </c>
+      <c r="B14" s="41" t="n">
+        <v>3</v>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>each</t>
+        </is>
+      </c>
+      <c r="D14" s="20" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E14" s="43" t="inlineStr">
+        <is>
+          <t>PURCHASED</t>
+        </is>
+      </c>
+      <c r="F14" s="24" t="n"/>
+      <c r="G14" s="24" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="12" t="inlineStr">
         <is>
           <t>At Dawn They Sleep - Batch</t>
         </is>
       </c>
-      <c r="C7" s="15" t="n">
+      <c r="B15" s="13" t="n"/>
+      <c r="C15" s="13" t="n"/>
+      <c r="D15" s="13" t="n"/>
+      <c r="E15" s="13" t="n"/>
+      <c r="F15" s="39" t="n">
         <v>25.48</v>
       </c>
-      <c r="D7" s="40" t="inlineStr">
+      <c r="G15" s="40" t="inlineStr">
         <is>
           <t>34 fl oz</t>
         </is>
       </c>
-      <c r="E7" s="41" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="39" t="n">
-        <v>328403264</v>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Grapefruit Infused Patron</t>
+        </is>
+      </c>
+      <c r="B16" s="41" t="n">
+        <v>11.25</v>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>fl oz</t>
+        </is>
+      </c>
+      <c r="D16" s="20" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="E16" s="45" t="inlineStr">
+        <is>
+          <t>SUBRECIPE</t>
+        </is>
+      </c>
+      <c r="F16" s="24" t="n"/>
+      <c r="G16" s="24" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Liqueur, Maggie's Farm Falernum</t>
+        </is>
+      </c>
+      <c r="B17" s="41" t="n">
+        <v>11.25</v>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>fl oz</t>
+        </is>
+      </c>
+      <c r="D17" s="20" t="n">
+        <v>14.61</v>
+      </c>
+      <c r="E17" s="42" t="inlineStr">
+        <is>
+          <t>SPIRIT</t>
+        </is>
+      </c>
+      <c r="F17" s="24" t="n"/>
+      <c r="G17" s="24" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Amaro Di Angostura</t>
+        </is>
+      </c>
+      <c r="B18" s="41" t="n">
+        <v>11.25</v>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>fl oz</t>
+        </is>
+      </c>
+      <c r="D18" s="20" t="n">
+        <v>10.84</v>
+      </c>
+      <c r="E18" s="42" t="inlineStr">
+        <is>
+          <t>SPIRIT</t>
+        </is>
+      </c>
+      <c r="F18" s="24" t="n"/>
+      <c r="G18" s="24" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="12" t="inlineStr">
         <is>
           <t>Bloody Mary Spice Blend</t>
         </is>
       </c>
-      <c r="C8" s="15" t="n">
+      <c r="B19" s="13" t="n"/>
+      <c r="C19" s="13" t="n"/>
+      <c r="D19" s="13" t="n"/>
+      <c r="E19" s="13" t="n"/>
+      <c r="F19" s="39" t="n">
         <v>1</v>
       </c>
-      <c r="D8" s="40" t="inlineStr">
+      <c r="G19" s="40" t="inlineStr">
         <is>
           <t>8.3 tbsp</t>
         </is>
       </c>
-      <c r="E8" s="41" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="39" t="n">
-        <v>333469888</v>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Spice, Celery Salt</t>
+        </is>
+      </c>
+      <c r="B20" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>tbsp</t>
+        </is>
+      </c>
+      <c r="D20" s="20" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E20" s="46" t="inlineStr">
+        <is>
+          <t>DRYSPICE</t>
+        </is>
+      </c>
+      <c r="F20" s="24" t="n"/>
+      <c r="G20" s="24" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Spice, Paprika (smoked)</t>
+        </is>
+      </c>
+      <c r="B21" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>tbsp</t>
+        </is>
+      </c>
+      <c r="D21" s="20" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="E21" s="46" t="inlineStr">
+        <is>
+          <t>DRYSPICE</t>
+        </is>
+      </c>
+      <c r="F21" s="24" t="n"/>
+      <c r="G21" s="24" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Spice, Chili Powder</t>
+        </is>
+      </c>
+      <c r="B22" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>tbsp</t>
+        </is>
+      </c>
+      <c r="D22" s="20" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="E22" s="46" t="inlineStr">
+        <is>
+          <t>DRYSPICE</t>
+        </is>
+      </c>
+      <c r="F22" s="24" t="n"/>
+      <c r="G22" s="24" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Spice, Onion Powder</t>
+        </is>
+      </c>
+      <c r="B23" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>tbsp</t>
+        </is>
+      </c>
+      <c r="D23" s="20" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="E23" s="46" t="inlineStr">
+        <is>
+          <t>DRYSPICE</t>
+        </is>
+      </c>
+      <c r="F23" s="24" t="n"/>
+      <c r="G23" s="24" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Spice, Cayenne Pepper</t>
+        </is>
+      </c>
+      <c r="B24" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>tbsp</t>
+        </is>
+      </c>
+      <c r="D24" s="20" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="E24" s="46" t="inlineStr">
+        <is>
+          <t>DRYSPICE</t>
+        </is>
+      </c>
+      <c r="F24" s="24" t="n"/>
+      <c r="G24" s="24" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Spice, Pepper Aleppo</t>
+        </is>
+      </c>
+      <c r="B25" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>tbsp</t>
+        </is>
+      </c>
+      <c r="D25" s="20" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="E25" s="46" t="inlineStr">
+        <is>
+          <t>DRYSPICE</t>
+        </is>
+      </c>
+      <c r="F25" s="24" t="n"/>
+      <c r="G25" s="24" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Oregano (dried)</t>
+        </is>
+      </c>
+      <c r="B26" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>tsp</t>
+        </is>
+      </c>
+      <c r="D26" s="20" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E26" s="46" t="inlineStr">
+        <is>
+          <t>DRYSPICE</t>
+        </is>
+      </c>
+      <c r="F26" s="24" t="n"/>
+      <c r="G26" s="24" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Spice, Cumin Ground</t>
+        </is>
+      </c>
+      <c r="B27" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>tsp</t>
+        </is>
+      </c>
+      <c r="D27" s="20" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="E27" s="46" t="inlineStr">
+        <is>
+          <t>DRYSPICE</t>
+        </is>
+      </c>
+      <c r="F27" s="24" t="n"/>
+      <c r="G27" s="24" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Spice, Pepper Black Ground</t>
+        </is>
+      </c>
+      <c r="B28" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>tsp</t>
+        </is>
+      </c>
+      <c r="D28" s="20" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="E28" s="46" t="inlineStr">
+        <is>
+          <t>DRYSPICE</t>
+        </is>
+      </c>
+      <c r="F28" s="24" t="n"/>
+      <c r="G28" s="24" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Dill (dried)</t>
+        </is>
+      </c>
+      <c r="B29" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>tsp</t>
+        </is>
+      </c>
+      <c r="D29" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" s="46" t="inlineStr">
+        <is>
+          <t>DRYSPICE</t>
+        </is>
+      </c>
+      <c r="F29" s="24" t="n"/>
+      <c r="G29" s="24" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="12" t="inlineStr">
         <is>
           <t>Brewed Chai Tea</t>
         </is>
       </c>
-      <c r="C9" s="15" t="n">
+      <c r="B30" s="13" t="n"/>
+      <c r="C30" s="13" t="n"/>
+      <c r="D30" s="13" t="n"/>
+      <c r="E30" s="13" t="n"/>
+      <c r="F30" s="39" t="n">
         <v>12.91</v>
       </c>
-      <c r="D9" s="40" t="inlineStr">
+      <c r="G30" s="40" t="inlineStr">
         <is>
           <t>32 fl oz</t>
         </is>
       </c>
-      <c r="E9" s="41" t="inlineStr">
-        <is>
-          <t>USES: Loose Leaf Chai 4 fl oz, Water 32 fl oz, Honey 2 fl oz</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="39" t="n">
-        <v>333468674</v>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Tea, Loose Leaf Chai</t>
+        </is>
+      </c>
+      <c r="B31" s="41" t="n">
+        <v>4</v>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>fl oz</t>
+        </is>
+      </c>
+      <c r="D31" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" s="43" t="inlineStr">
+        <is>
+          <t>PURCHASED</t>
+        </is>
+      </c>
+      <c r="F31" s="24" t="n"/>
+      <c r="G31" s="24" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Water</t>
+        </is>
+      </c>
+      <c r="B32" s="41" t="n">
+        <v>32</v>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>fl oz</t>
+        </is>
+      </c>
+      <c r="D32" s="20" t="n">
+        <v>12.28</v>
+      </c>
+      <c r="E32" s="44" t="inlineStr">
+        <is>
+          <t>WATER</t>
+        </is>
+      </c>
+      <c r="F32" s="24" t="n"/>
+      <c r="G32" s="24" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Honey</t>
+        </is>
+      </c>
+      <c r="B33" s="41" t="n">
+        <v>2</v>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>fl oz</t>
+        </is>
+      </c>
+      <c r="D33" s="20" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="E33" s="43" t="inlineStr">
+        <is>
+          <t>PURCHASED</t>
+        </is>
+      </c>
+      <c r="F33" s="24" t="n"/>
+      <c r="G33" s="24" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="12" t="inlineStr">
         <is>
           <t>Channel Orange - Batched</t>
         </is>
       </c>
-      <c r="C10" s="15" t="n">
+      <c r="B34" s="13" t="n"/>
+      <c r="C34" s="13" t="n"/>
+      <c r="D34" s="13" t="n"/>
+      <c r="E34" s="13" t="n"/>
+      <c r="F34" s="39" t="n">
         <v>30.78</v>
       </c>
-      <c r="D10" s="40" t="inlineStr">
+      <c r="G34" s="40" t="inlineStr">
         <is>
           <t>32 fl oz</t>
         </is>
       </c>
-      <c r="E10" s="41" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="39" t="n">
-        <v>333464610</v>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Gin, Malfy Con Arancia</t>
+        </is>
+      </c>
+      <c r="B35" s="41" t="n">
+        <v>29</v>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>fl oz</t>
+        </is>
+      </c>
+      <c r="D35" s="20" t="n">
+        <v>26.84</v>
+      </c>
+      <c r="E35" s="42" t="inlineStr">
+        <is>
+          <t>SPIRIT</t>
+        </is>
+      </c>
+      <c r="F35" s="24" t="n"/>
+      <c r="G35" s="24" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Liqueur, St. Elder Elderflower</t>
+        </is>
+      </c>
+      <c r="B36" s="41" t="n">
+        <v>4.75</v>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>fl oz</t>
+        </is>
+      </c>
+      <c r="D36" s="20" t="n">
+        <v>3.93</v>
+      </c>
+      <c r="E36" s="42" t="inlineStr">
+        <is>
+          <t>SPIRIT</t>
+        </is>
+      </c>
+      <c r="F36" s="24" t="n"/>
+      <c r="G36" s="24" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Bitters, Orange</t>
+        </is>
+      </c>
+      <c r="B37" s="41" t="n">
+        <v>2</v>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>tsp</t>
+        </is>
+      </c>
+      <c r="D37" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="E37" s="43" t="inlineStr">
+        <is>
+          <t>PURCHASED</t>
+        </is>
+      </c>
+      <c r="F37" s="24" t="n"/>
+      <c r="G37" s="24" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="12" t="inlineStr">
         <is>
           <t>Crash Course - Batched</t>
         </is>
       </c>
-      <c r="C11" s="15" t="n">
+      <c r="B38" s="13" t="n"/>
+      <c r="C38" s="13" t="n"/>
+      <c r="D38" s="13" t="n"/>
+      <c r="E38" s="13" t="n"/>
+      <c r="F38" s="39" t="n">
         <v>26.19</v>
       </c>
-      <c r="D11" s="40" t="inlineStr">
+      <c r="G38" s="40" t="inlineStr">
         <is>
           <t>32 fl oz</t>
         </is>
       </c>
-      <c r="E11" s="41" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="39" t="n">
-        <v>333504278</v>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Syrup, Queen of Earl</t>
+        </is>
+      </c>
+      <c r="B39" s="41" t="n">
+        <v>5</v>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>fl oz</t>
+        </is>
+      </c>
+      <c r="D39" s="20" t="n">
+        <v>1.97</v>
+      </c>
+      <c r="E39" s="45" t="inlineStr">
+        <is>
+          <t>SUBRECIPE</t>
+        </is>
+      </c>
+      <c r="F39" s="24" t="n"/>
+      <c r="G39" s="24" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Amaro Montenegro</t>
+        </is>
+      </c>
+      <c r="B40" s="41" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>fl oz</t>
+        </is>
+      </c>
+      <c r="D40" s="20" t="n">
+        <v>3.71</v>
+      </c>
+      <c r="E40" s="42" t="inlineStr">
+        <is>
+          <t>SPIRIT</t>
+        </is>
+      </c>
+      <c r="F40" s="24" t="n"/>
+      <c r="G40" s="24" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Bourbon, George Dickel Rye</t>
+        </is>
+      </c>
+      <c r="B41" s="41" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>fl oz</t>
+        </is>
+      </c>
+      <c r="D41" s="20" t="n">
+        <v>18.35</v>
+      </c>
+      <c r="E41" s="42" t="inlineStr">
+        <is>
+          <t>SPIRIT</t>
+        </is>
+      </c>
+      <c r="F41" s="24" t="n"/>
+      <c r="G41" s="24" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Bitters, Xocolatl Mole</t>
+        </is>
+      </c>
+      <c r="B42" s="41" t="n">
+        <v>4</v>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>each</t>
+        </is>
+      </c>
+      <c r="D42" s="20" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="E42" s="43" t="inlineStr">
+        <is>
+          <t>PURCHASED</t>
+        </is>
+      </c>
+      <c r="F42" s="24" t="n"/>
+      <c r="G42" s="24" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Bitters, Barkeep Lavender</t>
+        </is>
+      </c>
+      <c r="B43" s="41" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>fl oz</t>
+        </is>
+      </c>
+      <c r="D43" s="20" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="E43" s="43" t="inlineStr">
+        <is>
+          <t>PURCHASED</t>
+        </is>
+      </c>
+      <c r="F43" s="24" t="n"/>
+      <c r="G43" s="24" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="12" t="inlineStr">
         <is>
           <t>Dragonwell Infused OYO Vodka</t>
         </is>
       </c>
-      <c r="C12" s="15" t="n">
+      <c r="B44" s="13" t="n"/>
+      <c r="C44" s="13" t="n"/>
+      <c r="D44" s="13" t="n"/>
+      <c r="E44" s="13" t="n"/>
+      <c r="F44" s="39" t="n">
         <v>16.45</v>
       </c>
-      <c r="D12" s="40" t="inlineStr">
+      <c r="G44" s="40" t="inlineStr">
         <is>
           <t>24 fl oz</t>
         </is>
       </c>
-      <c r="E12" s="41" t="inlineStr">
-        <is>
-          <t>Spirit infusion — liquor vendor</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="39" t="n">
-        <v>333500998</v>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Vodka, OYO</t>
+        </is>
+      </c>
+      <c r="B45" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>bottle</t>
+        </is>
+      </c>
+      <c r="D45" s="20" t="n">
+        <v>16.45</v>
+      </c>
+      <c r="E45" s="42" t="inlineStr">
+        <is>
+          <t>SPIRIT</t>
+        </is>
+      </c>
+      <c r="F45" s="24" t="n"/>
+      <c r="G45" s="24" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="12" t="inlineStr">
         <is>
           <t>Espresso Martini Mix</t>
         </is>
       </c>
-      <c r="C13" s="15" t="n">
+      <c r="B46" s="13" t="n"/>
+      <c r="C46" s="13" t="n"/>
+      <c r="D46" s="13" t="n"/>
+      <c r="E46" s="13" t="n"/>
+      <c r="F46" s="39" t="n">
         <v>3.8</v>
       </c>
-      <c r="D13" s="40" t="inlineStr">
+      <c r="G46" s="40" t="inlineStr">
         <is>
           <t>25.4 fl oz</t>
         </is>
       </c>
-      <c r="E13" s="41" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="39" t="n">
-        <v>333492968</v>
-      </c>
-      <c r="B14" s="4" t="inlineStr">
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Espresso Shot</t>
+        </is>
+      </c>
+      <c r="B47" s="41" t="n">
+        <v>12.7</v>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>fl oz</t>
+        </is>
+      </c>
+      <c r="D47" s="20" t="n">
+        <v>1.94</v>
+      </c>
+      <c r="E47" s="45" t="inlineStr">
+        <is>
+          <t>SUBRECIPE</t>
+        </is>
+      </c>
+      <c r="F47" s="24" t="n"/>
+      <c r="G47" s="24" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Six Shooter Cold Brew Gal</t>
+        </is>
+      </c>
+      <c r="B48" s="41" t="n">
+        <v>12.7</v>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>fl oz</t>
+        </is>
+      </c>
+      <c r="D48" s="20" t="n">
+        <v>1.86</v>
+      </c>
+      <c r="E48" s="43" t="inlineStr">
+        <is>
+          <t>PURCHASED</t>
+        </is>
+      </c>
+      <c r="F48" s="24" t="n"/>
+      <c r="G48" s="24" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="12" t="inlineStr">
         <is>
           <t>Fall Coconut Cream</t>
         </is>
       </c>
-      <c r="C14" s="15" t="n">
+      <c r="B49" s="13" t="n"/>
+      <c r="C49" s="13" t="n"/>
+      <c r="D49" s="13" t="n"/>
+      <c r="E49" s="13" t="n"/>
+      <c r="F49" s="39" t="n">
         <v>18.14</v>
       </c>
-      <c r="D14" s="40" t="inlineStr">
+      <c r="G49" s="40" t="inlineStr">
         <is>
           <t>72 fl oz</t>
         </is>
       </c>
-      <c r="E14" s="41" t="inlineStr">
-        <is>
-          <t>USES: Coconut Cream 15 fl oz, Coconut Milk 13.5 fl oz, pineapple, allspice, cinnamon, nutmeg, pom molasses</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="39" t="n">
-        <v>333473987</v>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Juice, Pineapple</t>
+        </is>
+      </c>
+      <c r="B50" s="41" t="n">
+        <v>22</v>
+      </c>
+      <c r="C50" s="4" t="inlineStr">
+        <is>
+          <t>fl oz</t>
+        </is>
+      </c>
+      <c r="D50" s="20" t="n">
+        <v>15.97</v>
+      </c>
+      <c r="E50" s="45" t="inlineStr">
+        <is>
+          <t>SUBRECIPE</t>
+        </is>
+      </c>
+      <c r="F50" s="24" t="n"/>
+      <c r="G50" s="24" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Coconut Cream</t>
+        </is>
+      </c>
+      <c r="B51" s="41" t="n">
+        <v>15</v>
+      </c>
+      <c r="C51" s="4" t="inlineStr">
+        <is>
+          <t>fl oz</t>
+        </is>
+      </c>
+      <c r="D51" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="E51" s="43" t="inlineStr">
+        <is>
+          <t>PURCHASED</t>
+        </is>
+      </c>
+      <c r="F51" s="24" t="n"/>
+      <c r="G51" s="24" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Milk, Coconut Canned</t>
+        </is>
+      </c>
+      <c r="B52" s="41" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="C52" s="4" t="inlineStr">
+        <is>
+          <t>fl oz</t>
+        </is>
+      </c>
+      <c r="D52" s="20" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="E52" s="43" t="inlineStr">
+        <is>
+          <t>PURCHASED</t>
+        </is>
+      </c>
+      <c r="F52" s="24" t="n"/>
+      <c r="G52" s="24" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Spice, Allspice Ground</t>
+        </is>
+      </c>
+      <c r="B53" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="C53" s="4" t="inlineStr">
+        <is>
+          <t>tsp</t>
+        </is>
+      </c>
+      <c r="D53" s="20" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="E53" s="46" t="inlineStr">
+        <is>
+          <t>DRYSPICE</t>
+        </is>
+      </c>
+      <c r="F53" s="24" t="n"/>
+      <c r="G53" s="24" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Spice, Cinnamon Ground</t>
+        </is>
+      </c>
+      <c r="B54" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="C54" s="4" t="inlineStr">
+        <is>
+          <t>tsp</t>
+        </is>
+      </c>
+      <c r="D54" s="20" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="E54" s="46" t="inlineStr">
+        <is>
+          <t>DRYSPICE</t>
+        </is>
+      </c>
+      <c r="F54" s="24" t="n"/>
+      <c r="G54" s="24" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Spice, Nutmeg Ground</t>
+        </is>
+      </c>
+      <c r="B55" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="C55" s="4" t="inlineStr">
+        <is>
+          <t>tsp</t>
+        </is>
+      </c>
+      <c r="D55" s="20" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="E55" s="46" t="inlineStr">
+        <is>
+          <t>DRYSPICE</t>
+        </is>
+      </c>
+      <c r="F55" s="24" t="n"/>
+      <c r="G55" s="24" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Molasses, Pomegranate</t>
+        </is>
+      </c>
+      <c r="B56" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="C56" s="4" t="inlineStr">
+        <is>
+          <t>tbsp</t>
+        </is>
+      </c>
+      <c r="D56" s="20" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="E56" s="43" t="inlineStr">
+        <is>
+          <t>PURCHASED</t>
+        </is>
+      </c>
+      <c r="F56" s="24" t="n"/>
+      <c r="G56" s="24" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="12" t="inlineStr">
         <is>
           <t>Grapefruit Infused Patron</t>
         </is>
       </c>
-      <c r="C15" s="15" t="n">
+      <c r="B57" s="13" t="n"/>
+      <c r="C57" s="13" t="n"/>
+      <c r="D57" s="13" t="n"/>
+      <c r="E57" s="13" t="n"/>
+      <c r="F57" s="39" t="n">
         <v>0.06</v>
       </c>
-      <c r="D15" s="40" t="inlineStr">
+      <c r="G57" s="40" t="inlineStr">
         <is>
           <t>1 bottle</t>
         </is>
       </c>
-      <c r="E15" s="41" t="inlineStr">
-        <is>
-          <t>Spirit infusion — cost looks wrong ($0.06)</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="39" t="n">
-        <v>333504038</v>
-      </c>
-      <c r="B16" s="4" t="inlineStr">
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Patron Silver</t>
+        </is>
+      </c>
+      <c r="B58" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="C58" s="4" t="inlineStr">
+        <is>
+          <t>bottle</t>
+        </is>
+      </c>
+      <c r="D58" s="20" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="E58" s="42" t="inlineStr">
+        <is>
+          <t>SPIRIT</t>
+        </is>
+      </c>
+      <c r="F58" s="24" t="n"/>
+      <c r="G58" s="24" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Grapefruit, Fresh (peel)</t>
+        </is>
+      </c>
+      <c r="B59" s="41" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C59" s="4" t="inlineStr">
+        <is>
+          <t>oz</t>
+        </is>
+      </c>
+      <c r="D59" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E59" s="48" t="inlineStr">
+        <is>
+          <t>PRODUCE</t>
+        </is>
+      </c>
+      <c r="F59" s="24" t="n"/>
+      <c r="G59" s="24" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="12" t="inlineStr">
         <is>
           <t>Green Goddess - Batch</t>
         </is>
       </c>
-      <c r="C16" s="15" t="n">
+      <c r="B60" s="13" t="n"/>
+      <c r="C60" s="13" t="n"/>
+      <c r="D60" s="13" t="n"/>
+      <c r="E60" s="13" t="n"/>
+      <c r="F60" s="39" t="n">
         <v>18.55</v>
       </c>
-      <c r="D16" s="40" t="inlineStr">
+      <c r="G60" s="40" t="inlineStr">
         <is>
           <t>33 fl oz</t>
         </is>
       </c>
-      <c r="E16" s="41" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="39" t="n">
-        <v>525737107</v>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
+    </row>
+    <row r="61">
+      <c r="A61" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Syrup, Arugula</t>
+        </is>
+      </c>
+      <c r="B61" s="41" t="n">
+        <v>9</v>
+      </c>
+      <c r="C61" s="4" t="inlineStr">
+        <is>
+          <t>fl oz</t>
+        </is>
+      </c>
+      <c r="D61" s="20" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="E61" s="45" t="inlineStr">
+        <is>
+          <t>SUBRECIPE</t>
+        </is>
+      </c>
+      <c r="F61" s="24" t="n"/>
+      <c r="G61" s="24" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Dragonwell Infused OYO Vodka</t>
+        </is>
+      </c>
+      <c r="B62" s="41" t="n">
+        <v>24</v>
+      </c>
+      <c r="C62" s="4" t="inlineStr">
+        <is>
+          <t>fl oz</t>
+        </is>
+      </c>
+      <c r="D62" s="20" t="n">
+        <v>16.45</v>
+      </c>
+      <c r="E62" s="45" t="inlineStr">
+        <is>
+          <t>SUBRECIPE</t>
+        </is>
+      </c>
+      <c r="F62" s="24" t="n"/>
+      <c r="G62" s="24" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="12" t="inlineStr">
         <is>
           <t>Heaven or LV BIZ - TH</t>
         </is>
       </c>
-      <c r="C17" s="15" t="n">
+      <c r="B63" s="13" t="n"/>
+      <c r="C63" s="13" t="n"/>
+      <c r="D63" s="13" t="n"/>
+      <c r="E63" s="13" t="n"/>
+      <c r="F63" s="39" t="n">
         <v>7.28</v>
       </c>
-      <c r="D17" s="40" t="inlineStr">
+      <c r="G63" s="40" t="inlineStr">
         <is>
           <t>4.5 fl oz</t>
         </is>
       </c>
-      <c r="E17" s="41" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="39" t="n">
-        <v>333481247</v>
-      </c>
-      <c r="B18" s="4" t="inlineStr">
+    </row>
+    <row r="64">
+      <c r="A64" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Cazadores Blanco Tequila</t>
+        </is>
+      </c>
+      <c r="B64" s="41" t="n">
+        <v>2</v>
+      </c>
+      <c r="C64" s="4" t="inlineStr">
+        <is>
+          <t>fl oz</t>
+        </is>
+      </c>
+      <c r="D64" s="20" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="E64" s="42" t="inlineStr">
+        <is>
+          <t>SPIRIT</t>
+        </is>
+      </c>
+      <c r="F64" s="24" t="n"/>
+      <c r="G64" s="24" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Honey</t>
+        </is>
+      </c>
+      <c r="B65" s="41" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C65" s="4" t="inlineStr">
+        <is>
+          <t>fl oz</t>
+        </is>
+      </c>
+      <c r="D65" s="20" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="E65" s="43" t="inlineStr">
+        <is>
+          <t>PURCHASED</t>
+        </is>
+      </c>
+      <c r="F65" s="24" t="n"/>
+      <c r="G65" s="24" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Juice, Lime</t>
+        </is>
+      </c>
+      <c r="B66" s="41" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="C66" s="4" t="inlineStr">
+        <is>
+          <t>fl oz</t>
+        </is>
+      </c>
+      <c r="D66" s="20" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="E66" s="43" t="inlineStr">
+        <is>
+          <t>PURCHASED</t>
+        </is>
+      </c>
+      <c r="F66" s="24" t="n"/>
+      <c r="G66" s="24" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Juice, Lemon</t>
+        </is>
+      </c>
+      <c r="B67" s="41" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="C67" s="4" t="inlineStr">
+        <is>
+          <t>fl oz</t>
+        </is>
+      </c>
+      <c r="D67" s="20" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="E67" s="43" t="inlineStr">
+        <is>
+          <t>PURCHASED</t>
+        </is>
+      </c>
+      <c r="F67" s="24" t="n"/>
+      <c r="G67" s="24" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Juice, Pineapple</t>
+        </is>
+      </c>
+      <c r="B68" s="41" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C68" s="4" t="inlineStr">
+        <is>
+          <t>fl oz</t>
+        </is>
+      </c>
+      <c r="D68" s="20" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="E68" s="43" t="inlineStr">
+        <is>
+          <t>PURCHASED</t>
+        </is>
+      </c>
+      <c r="F68" s="24" t="n"/>
+      <c r="G68" s="24" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Tea, Butterfly Pea Flowers</t>
+        </is>
+      </c>
+      <c r="B69" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="C69" s="4" t="inlineStr">
+        <is>
+          <t>oz</t>
+        </is>
+      </c>
+      <c r="D69" s="20" t="n">
+        <v>5.45</v>
+      </c>
+      <c r="E69" s="43" t="inlineStr">
+        <is>
+          <t>PURCHASED</t>
+        </is>
+      </c>
+      <c r="F69" s="24" t="n"/>
+      <c r="G69" s="24" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="12" t="inlineStr">
         <is>
           <t>Jammy Pom Juice</t>
         </is>
       </c>
-      <c r="C18" s="15" t="n">
+      <c r="B70" s="13" t="n"/>
+      <c r="C70" s="13" t="n"/>
+      <c r="D70" s="13" t="n"/>
+      <c r="E70" s="13" t="n"/>
+      <c r="F70" s="39" t="n">
         <v>8.199999999999999</v>
       </c>
-      <c r="D18" s="40" t="inlineStr">
+      <c r="G70" s="40" t="inlineStr">
         <is>
           <t>35 fl oz</t>
         </is>
       </c>
-      <c r="E18" s="41" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="39" t="n">
-        <v>333486093</v>
-      </c>
-      <c r="B19" s="4" t="inlineStr">
+    </row>
+    <row r="71">
+      <c r="A71" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Juice, Pomegranate</t>
+        </is>
+      </c>
+      <c r="B71" s="41" t="n">
+        <v>20</v>
+      </c>
+      <c r="C71" s="4" t="inlineStr">
+        <is>
+          <t>fl oz</t>
+        </is>
+      </c>
+      <c r="D71" s="20" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="E71" s="43" t="inlineStr">
+        <is>
+          <t>PURCHASED</t>
+        </is>
+      </c>
+      <c r="F71" s="24" t="n"/>
+      <c r="G71" s="24" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Juice, Grapefruit</t>
+        </is>
+      </c>
+      <c r="B72" s="41" t="n">
+        <v>10</v>
+      </c>
+      <c r="C72" s="4" t="inlineStr">
+        <is>
+          <t>fl oz</t>
+        </is>
+      </c>
+      <c r="D72" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E72" s="45" t="inlineStr">
+        <is>
+          <t>SUBRECIPE</t>
+        </is>
+      </c>
+      <c r="F72" s="24" t="n"/>
+      <c r="G72" s="24" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Preserves, Lingonberry</t>
+        </is>
+      </c>
+      <c r="B73" s="41" t="n">
+        <v>5</v>
+      </c>
+      <c r="C73" s="4" t="inlineStr">
+        <is>
+          <t>fl oz</t>
+        </is>
+      </c>
+      <c r="D73" s="20" t="n">
+        <v>3.14</v>
+      </c>
+      <c r="E73" s="43" t="inlineStr">
+        <is>
+          <t>PURCHASED</t>
+        </is>
+      </c>
+      <c r="F73" s="24" t="n"/>
+      <c r="G73" s="24" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Jelly, Hot Pepper</t>
+        </is>
+      </c>
+      <c r="B74" s="41" t="n">
+        <v>5</v>
+      </c>
+      <c r="C74" s="4" t="inlineStr">
+        <is>
+          <t>fl oz</t>
+        </is>
+      </c>
+      <c r="D74" s="20" t="n">
+        <v>1.94</v>
+      </c>
+      <c r="E74" s="43" t="inlineStr">
+        <is>
+          <t>PURCHASED</t>
+        </is>
+      </c>
+      <c r="F74" s="24" t="n"/>
+      <c r="G74" s="24" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="12" t="inlineStr">
         <is>
           <t>Lemony Lemon Curd Juice</t>
         </is>
       </c>
-      <c r="C19" s="15" t="n">
+      <c r="B75" s="13" t="n"/>
+      <c r="C75" s="13" t="n"/>
+      <c r="D75" s="13" t="n"/>
+      <c r="E75" s="13" t="n"/>
+      <c r="F75" s="39" t="n">
         <v>2.42</v>
       </c>
-      <c r="D19" s="40" t="inlineStr">
+      <c r="G75" s="40" t="inlineStr">
         <is>
           <t>25 fl oz</t>
         </is>
       </c>
-      <c r="E19" s="41" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="39" t="n">
-        <v>333470550</v>
-      </c>
-      <c r="B20" s="4" t="inlineStr">
+    </row>
+    <row r="76">
+      <c r="A76" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Juice, Lemon</t>
+        </is>
+      </c>
+      <c r="B76" s="41" t="n">
+        <v>20</v>
+      </c>
+      <c r="C76" s="4" t="inlineStr">
+        <is>
+          <t>fl oz</t>
+        </is>
+      </c>
+      <c r="D76" s="20" t="n">
+        <v>2.42</v>
+      </c>
+      <c r="E76" s="43" t="inlineStr">
+        <is>
+          <t>PURCHASED</t>
+        </is>
+      </c>
+      <c r="F76" s="24" t="n"/>
+      <c r="G76" s="24" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Preserves, Lemon Curd</t>
+        </is>
+      </c>
+      <c r="B77" s="41" t="n">
+        <v>5</v>
+      </c>
+      <c r="C77" s="4" t="inlineStr">
+        <is>
+          <t>fl oz</t>
+        </is>
+      </c>
+      <c r="D77" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="E77" s="43" t="inlineStr">
+        <is>
+          <t>PURCHASED</t>
+        </is>
+      </c>
+      <c r="F77" s="24" t="n"/>
+      <c r="G77" s="24" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="12" t="inlineStr">
         <is>
           <t>Pear Chai Tea</t>
         </is>
       </c>
-      <c r="C20" s="15" t="n">
+      <c r="B78" s="13" t="n"/>
+      <c r="C78" s="13" t="n"/>
+      <c r="D78" s="13" t="n"/>
+      <c r="E78" s="13" t="n"/>
+      <c r="F78" s="39" t="n">
         <v>8.880000000000001</v>
       </c>
-      <c r="D20" s="40" t="inlineStr">
+      <c r="G78" s="40" t="inlineStr">
         <is>
           <t>34 fl oz</t>
         </is>
       </c>
-      <c r="E20" s="41" t="inlineStr">
-        <is>
-          <t>USES: Pear Simple Syrup, Brewed Chai Tea, Lemon Juice</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="39" t="n">
-        <v>333504478</v>
-      </c>
-      <c r="B21" s="4" t="inlineStr">
+    </row>
+    <row r="79">
+      <c r="A79" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Syrup, Pear Simple</t>
+        </is>
+      </c>
+      <c r="B79" s="41" t="n">
+        <v>11.25</v>
+      </c>
+      <c r="C79" s="4" t="inlineStr">
+        <is>
+          <t>fl oz</t>
+        </is>
+      </c>
+      <c r="D79" s="20" t="n">
+        <v>2.98</v>
+      </c>
+      <c r="E79" s="45" t="inlineStr">
+        <is>
+          <t>SUBRECIPE</t>
+        </is>
+      </c>
+      <c r="F79" s="24" t="n"/>
+      <c r="G79" s="24" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Brewed Chai Tea</t>
+        </is>
+      </c>
+      <c r="B80" s="41" t="n">
+        <v>11.25</v>
+      </c>
+      <c r="C80" s="4" t="inlineStr">
+        <is>
+          <t>fl oz</t>
+        </is>
+      </c>
+      <c r="D80" s="20" t="n">
+        <v>4.54</v>
+      </c>
+      <c r="E80" s="45" t="inlineStr">
+        <is>
+          <t>SUBRECIPE</t>
+        </is>
+      </c>
+      <c r="F80" s="24" t="n"/>
+      <c r="G80" s="24" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Juice, Lemon</t>
+        </is>
+      </c>
+      <c r="B81" s="41" t="n">
+        <v>11.25</v>
+      </c>
+      <c r="C81" s="4" t="inlineStr">
+        <is>
+          <t>fl oz</t>
+        </is>
+      </c>
+      <c r="D81" s="20" t="n">
+        <v>1.36</v>
+      </c>
+      <c r="E81" s="43" t="inlineStr">
+        <is>
+          <t>PURCHASED</t>
+        </is>
+      </c>
+      <c r="F81" s="24" t="n"/>
+      <c r="G81" s="24" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="12" t="inlineStr">
         <is>
           <t>Spicy Cucumber Juice</t>
         </is>
       </c>
-      <c r="C21" s="15" t="n">
+      <c r="B82" s="13" t="n"/>
+      <c r="C82" s="13" t="n"/>
+      <c r="D82" s="13" t="n"/>
+      <c r="E82" s="13" t="n"/>
+      <c r="F82" s="39" t="n">
         <v>7.18</v>
       </c>
-      <c r="D21" s="40" t="inlineStr">
+      <c r="G82" s="40" t="inlineStr">
         <is>
           <t>33.25 fl oz</t>
         </is>
       </c>
-      <c r="E21" s="41" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="39" t="n">
-        <v>333485862</v>
-      </c>
-      <c r="B22" s="4" t="inlineStr">
+    </row>
+    <row r="83">
+      <c r="A83" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Juice, Cucumber</t>
+        </is>
+      </c>
+      <c r="B83" s="41" t="n">
+        <v>33</v>
+      </c>
+      <c r="C83" s="4" t="inlineStr">
+        <is>
+          <t>fl oz</t>
+        </is>
+      </c>
+      <c r="D83" s="20" t="n">
+        <v>7.15</v>
+      </c>
+      <c r="E83" s="45" t="inlineStr">
+        <is>
+          <t>SUBRECIPE</t>
+        </is>
+      </c>
+      <c r="F83" s="24" t="n"/>
+      <c r="G83" s="24" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Juice, Jalapeno</t>
+        </is>
+      </c>
+      <c r="B84" s="41" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="C84" s="4" t="inlineStr">
+        <is>
+          <t>fl oz</t>
+        </is>
+      </c>
+      <c r="D84" s="20" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="E84" s="45" t="inlineStr">
+        <is>
+          <t>SUBRECIPE</t>
+        </is>
+      </c>
+      <c r="F84" s="24" t="n"/>
+      <c r="G84" s="24" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="12" t="inlineStr">
         <is>
           <t>Strawberry Infused Bombay Bramble</t>
         </is>
       </c>
-      <c r="C22" s="15" t="n">
+      <c r="B85" s="13" t="n"/>
+      <c r="C85" s="13" t="n"/>
+      <c r="D85" s="13" t="n"/>
+      <c r="E85" s="13" t="n"/>
+      <c r="F85" s="39" t="n">
         <v>22.33</v>
       </c>
-      <c r="D22" s="40" t="inlineStr">
+      <c r="G85" s="40" t="inlineStr">
         <is>
           <t>24.5 fl oz</t>
         </is>
       </c>
-      <c r="E22" s="41" t="inlineStr">
-        <is>
-          <t>Spirit infusion — liquor vendor</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="39" t="n">
-        <v>333486498</v>
-      </c>
-      <c r="B23" s="4" t="inlineStr">
+    </row>
+    <row r="86">
+      <c r="A86" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Bombay Bramble</t>
+        </is>
+      </c>
+      <c r="B86" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="C86" s="4" t="inlineStr">
+        <is>
+          <t>bottle</t>
+        </is>
+      </c>
+      <c r="D86" s="20" t="n">
+        <v>20.68</v>
+      </c>
+      <c r="E86" s="42" t="inlineStr">
+        <is>
+          <t>SPIRIT</t>
+        </is>
+      </c>
+      <c r="F86" s="24" t="n"/>
+      <c r="G86" s="24" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Strawberries, Fresh</t>
+        </is>
+      </c>
+      <c r="B87" s="41" t="n">
+        <v>120</v>
+      </c>
+      <c r="C87" s="4" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="D87" s="20" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="E87" s="48" t="inlineStr">
+        <is>
+          <t>PRODUCE</t>
+        </is>
+      </c>
+      <c r="F87" s="24" t="n"/>
+      <c r="G87" s="24" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="12" t="inlineStr">
         <is>
           <t>Strawberry Kush - Batch</t>
         </is>
       </c>
-      <c r="C23" s="15" t="n">
+      <c r="B88" s="13" t="n"/>
+      <c r="C88" s="13" t="n"/>
+      <c r="D88" s="13" t="n"/>
+      <c r="E88" s="13" t="n"/>
+      <c r="F88" s="39" t="n">
         <v>33.51</v>
       </c>
-      <c r="D23" s="40" t="inlineStr">
+      <c r="G88" s="40" t="inlineStr">
         <is>
           <t>40 fl oz</t>
         </is>
       </c>
-      <c r="E23" s="41" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="39" t="n">
-        <v>333498796</v>
-      </c>
-      <c r="B24" s="4" t="inlineStr">
+    </row>
+    <row r="89">
+      <c r="A89" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Strawberry Infused Bombay Bramble</t>
+        </is>
+      </c>
+      <c r="B89" s="41" t="n">
+        <v>28.2</v>
+      </c>
+      <c r="C89" s="4" t="inlineStr">
+        <is>
+          <t>fl oz</t>
+        </is>
+      </c>
+      <c r="D89" s="20" t="n">
+        <v>25.71</v>
+      </c>
+      <c r="E89" s="45" t="inlineStr">
+        <is>
+          <t>SUBRECIPE</t>
+        </is>
+      </c>
+      <c r="F89" s="24" t="n"/>
+      <c r="G89" s="24" t="n"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Syrup, Orgeat</t>
+        </is>
+      </c>
+      <c r="B90" s="41" t="n">
+        <v>11</v>
+      </c>
+      <c r="C90" s="4" t="inlineStr">
+        <is>
+          <t>fl oz</t>
+        </is>
+      </c>
+      <c r="D90" s="20" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="E90" s="43" t="inlineStr">
+        <is>
+          <t>PURCHASED</t>
+        </is>
+      </c>
+      <c r="F90" s="24" t="n"/>
+      <c r="G90" s="24" t="n"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Bitters, Toasted Almond</t>
+        </is>
+      </c>
+      <c r="B91" s="41" t="n">
+        <v>2</v>
+      </c>
+      <c r="C91" s="4" t="inlineStr">
+        <is>
+          <t>tsp</t>
+        </is>
+      </c>
+      <c r="D91" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="E91" s="43" t="inlineStr">
+        <is>
+          <t>PURCHASED</t>
+        </is>
+      </c>
+      <c r="F91" s="24" t="n"/>
+      <c r="G91" s="24" t="n"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="12" t="inlineStr">
         <is>
           <t>Sweetheart Infused Vodka</t>
         </is>
       </c>
-      <c r="C24" s="15" t="n">
+      <c r="B92" s="13" t="n"/>
+      <c r="C92" s="13" t="n"/>
+      <c r="D92" s="13" t="n"/>
+      <c r="E92" s="13" t="n"/>
+      <c r="F92" s="39" t="n">
         <v>19.72</v>
       </c>
-      <c r="D24" s="40" t="inlineStr">
+      <c r="G92" s="40" t="inlineStr">
         <is>
           <t>27 fl oz</t>
         </is>
       </c>
-      <c r="E24" s="41" t="inlineStr">
-        <is>
-          <t>Spirit infusion — liquor vendor</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="39" t="n">
-        <v>333504145</v>
-      </c>
-      <c r="B25" s="4" t="inlineStr">
+    </row>
+    <row r="93">
+      <c r="A93" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Absolut Vodka</t>
+        </is>
+      </c>
+      <c r="B93" s="41" t="n">
+        <v>25</v>
+      </c>
+      <c r="C93" s="4" t="inlineStr">
+        <is>
+          <t>fl oz</t>
+        </is>
+      </c>
+      <c r="D93" s="20" t="n">
+        <v>14.11</v>
+      </c>
+      <c r="E93" s="42" t="inlineStr">
+        <is>
+          <t>SPIRIT</t>
+        </is>
+      </c>
+      <c r="F93" s="24" t="n"/>
+      <c r="G93" s="24" t="n"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Strawberries, Fresh</t>
+        </is>
+      </c>
+      <c r="B94" s="41" t="n">
+        <v>240</v>
+      </c>
+      <c r="C94" s="4" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="D94" s="20" t="n">
+        <v>3.24</v>
+      </c>
+      <c r="E94" s="48" t="inlineStr">
+        <is>
+          <t>PRODUCE</t>
+        </is>
+      </c>
+      <c r="F94" s="24" t="n"/>
+      <c r="G94" s="24" t="n"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Tea, Peruvian Spiced Berry</t>
+        </is>
+      </c>
+      <c r="B95" s="41" t="n">
+        <v>2</v>
+      </c>
+      <c r="C95" s="4" t="inlineStr">
+        <is>
+          <t>oz</t>
+        </is>
+      </c>
+      <c r="D95" s="20" t="n">
+        <v>2.38</v>
+      </c>
+      <c r="E95" s="43" t="inlineStr">
+        <is>
+          <t>PURCHASED</t>
+        </is>
+      </c>
+      <c r="F95" s="24" t="n"/>
+      <c r="G95" s="24" t="n"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="12" t="inlineStr">
         <is>
           <t>Syrup, Arugula</t>
         </is>
       </c>
-      <c r="C25" s="15" t="n">
+      <c r="B96" s="13" t="n"/>
+      <c r="C96" s="13" t="n"/>
+      <c r="D96" s="13" t="n"/>
+      <c r="E96" s="13" t="n"/>
+      <c r="F96" s="39" t="n">
         <v>2.8</v>
       </c>
-      <c r="D25" s="40" t="inlineStr">
+      <c r="G96" s="40" t="inlineStr">
         <is>
           <t>12 fl oz</t>
         </is>
       </c>
-      <c r="E25" s="41" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="39" t="n">
-        <v>333468799</v>
-      </c>
-      <c r="B26" s="4" t="inlineStr">
+    </row>
+    <row r="97">
+      <c r="A97" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Simple Syrup</t>
+        </is>
+      </c>
+      <c r="B97" s="41" t="n">
+        <v>8</v>
+      </c>
+      <c r="C97" s="4" t="inlineStr">
+        <is>
+          <t>fl oz</t>
+        </is>
+      </c>
+      <c r="D97" s="20" t="n">
+        <v>2.26</v>
+      </c>
+      <c r="E97" s="45" t="inlineStr">
+        <is>
+          <t>SUBRECIPE</t>
+        </is>
+      </c>
+      <c r="F97" s="24" t="n"/>
+      <c r="G97" s="24" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Arugula, Baby</t>
+        </is>
+      </c>
+      <c r="B98" s="41" t="n">
+        <v>2</v>
+      </c>
+      <c r="C98" s="4" t="inlineStr">
+        <is>
+          <t>cup</t>
+        </is>
+      </c>
+      <c r="D98" s="20" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="E98" s="48" t="inlineStr">
+        <is>
+          <t>PRODUCE</t>
+        </is>
+      </c>
+      <c r="F98" s="24" t="n"/>
+      <c r="G98" s="24" t="n"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="12" t="inlineStr">
         <is>
           <t>Syrup, Pear Simple</t>
         </is>
       </c>
-      <c r="C26" s="15" t="n">
+      <c r="B99" s="13" t="n"/>
+      <c r="C99" s="13" t="n"/>
+      <c r="D99" s="13" t="n"/>
+      <c r="E99" s="13" t="n"/>
+      <c r="F99" s="39" t="n">
         <v>8.470000000000001</v>
       </c>
-      <c r="D26" s="40" t="inlineStr">
+      <c r="G99" s="40" t="inlineStr">
         <is>
           <t>32 fl oz</t>
         </is>
       </c>
-      <c r="E26" s="41" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="39" t="n">
-        <v>333460643</v>
-      </c>
-      <c r="B27" s="4" t="inlineStr">
+    </row>
+    <row r="100">
+      <c r="A100" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Simple Syrup</t>
+        </is>
+      </c>
+      <c r="B100" s="41" t="n">
+        <v>25</v>
+      </c>
+      <c r="C100" s="4" t="inlineStr">
+        <is>
+          <t>fl oz</t>
+        </is>
+      </c>
+      <c r="D100" s="20" t="n">
+        <v>7.07</v>
+      </c>
+      <c r="E100" s="45" t="inlineStr">
+        <is>
+          <t>SUBRECIPE</t>
+        </is>
+      </c>
+      <c r="F100" s="24" t="n"/>
+      <c r="G100" s="24" t="n"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Pears, Fresh</t>
+        </is>
+      </c>
+      <c r="B101" s="41" t="n">
+        <v>4</v>
+      </c>
+      <c r="C101" s="4" t="inlineStr">
+        <is>
+          <t>each</t>
+        </is>
+      </c>
+      <c r="D101" s="20" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="E101" s="48" t="inlineStr">
+        <is>
+          <t>PRODUCE</t>
+        </is>
+      </c>
+      <c r="F101" s="24" t="n"/>
+      <c r="G101" s="24" t="n"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="12" t="inlineStr">
         <is>
           <t>Syrup, Queen of Earl</t>
         </is>
       </c>
-      <c r="C27" s="15" t="n">
+      <c r="B102" s="13" t="n"/>
+      <c r="C102" s="13" t="n"/>
+      <c r="D102" s="13" t="n"/>
+      <c r="E102" s="13" t="n"/>
+      <c r="F102" s="39" t="n">
         <v>6.3</v>
       </c>
-      <c r="D27" s="40" t="inlineStr">
+      <c r="G102" s="40" t="inlineStr">
         <is>
           <t>16 fl oz</t>
         </is>
       </c>
-      <c r="E27" s="41" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="9" t="inlineStr">
-        <is>
-          <t>Only 3 of the 23 had their ingredient lists pulled (noted above). Hibiscus syrups sit under 'TH - Prep', not 'TH - Bar Prep'.</t>
+    </row>
+    <row r="103">
+      <c r="A103" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Sugar, Demerara</t>
+        </is>
+      </c>
+      <c r="B103" s="41" t="n">
+        <v>454</v>
+      </c>
+      <c r="C103" s="4" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="D103" s="20" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="E103" s="43" t="inlineStr">
+        <is>
+          <t>PURCHASED</t>
+        </is>
+      </c>
+      <c r="F103" s="24" t="n"/>
+      <c r="G103" s="24" t="n"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="49" t="inlineStr">
+        <is>
+          <t>ERRORS VISIBLE HERE:</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - Grapefruit Infused Patron: a bottle of Patron Silver is costed at $0.06. Should be roughly $45-50.</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - Water is costed at Columbus in 2 bar recipes ($12.28 / 32 fl oz and $5.85 / 15.25 fl oz). Cleveland charges $0.00.</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - Four purchased goods are costed at $0.00: Coconut Cream, Tea Loose Leaf Chai, Preserves Lemon Curd, Bitters Orange, Bitters Toasted Almond.</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - Together these understate bar prep costs; the water entries overstate them.</t>
         </is>
       </c>
     </row>

</xml_diff>